<commit_message>
Fill Kupishuz answers from the Lamoda interview.
Krylatskaya recordings are Lamoda, not Areal. The company file and the summary column now use those answers, and Areal no longer includes Lamoda-only details.

Co-authored-by: lysakalenushka-hash <lysakalenushka-hash@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/транскрипции/Ответы по вопросам/Сводная по интервью ЭДО.xlsx
+++ b/транскрипции/Ответы по вопросам/Сводная по интервью ЭДО.xlsx
@@ -69,12 +69,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4F4F4"/>
+        <fgColor rgb="00F7FBFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F7FBFF"/>
+        <fgColor rgb="00F4F4F4"/>
       </patternFill>
     </fill>
   </fills>
@@ -118,11 +118,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -554,7 +554,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>КУПИШУЗ</t>
+          <t>КУПИШУЗ (Ламода)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -580,7 +580,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Кржижановский и коллеги со стороны охраны труда показывают, как на предприятиях устроены ознакомление, подписание и учёт, и обсуждают выбор системы. Личный перечень документов и формальное участие во внедрении конкретной СЭД в записи не названы: компания на этапе выбора системы и описания процессов верхнего уровня. В разговоре рядом кадры (блоки документов при приёме и переводе), информационная безопасность, площадки и горные мастера, а также внешние контуры обучения и спецоценки.</t>
+          <t>Кржижановский и коллеги со стороны охраны труда показывают, как на предприятиях устроены ознакомление, подписание и учёт, и обсуждают выбор системы. Личный перечень документов и формальное участие во внедрении конкретной СЭД в записи не названы: компания на этапе выбора системы и описания процессов верхнего уровня. В разговоре рядом информационная безопасность, площадки и горные мастера, а также внешние контуры обучения и спецоценки.</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -603,9 +603,9 @@
           <t>Собеседник ведёт охрану труда по электростанциям и филиалам и говорит от первого лица про мобильное приложение, наряды-допуски и решение не отказываться от бумаги. Имя в записи не слышно. В выборе «уйти с бумаги целиком» ключ, по его словам, у первого лица: надо принять ответственность. С информационной безопасностью он согласовывал вход в приложение. Учебный центр, филиалы, в том числе Кольский, и подрядчики в записи есть. Кадрового ЭДО у них нет, и это не его внедрение.</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Позднякова говорит со стороны охраны труда. В записи к ней обращаются «Насть», компанию в начале называют «Ломода». Её зона в разговоре — инструкции для пунктов выдачи, протоколы проверки знаний, ознакомление в КЭДО и личные карточки по охране труда. Насколько она сама выбирала систему, не сказано. Рядом проектная команда по карточкам, кадры (блоки документов при приёме и переводе), руководители, которые заводят первичный и повторный инструктаж, и кладовщики: объектов много, фраза про кладовщика обрывается.</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -629,37 +629,37 @@
 Уточнения: Когда это началось? С каких документов начали? Почему начали именно с них? Кто выступил инициатором? Что стало причиной внедрения? Было ли это отдельное решение службы ОТ или часть общей цифровизации организации?</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Точный год старта и инициатор не названы. Уже есть подписание приказов и ознакомление в КЭДО. Личные карточки по охране труда в электронный документооборот ещё не переведены целиком, этим занимается проектная команда; электронное подписание, по их словам, только стартует, а целевая доля — 100%. Причина, которая звучит: объём бумаги и ознакомлений (на разных предприятиях от 21 до 45 документов на человека), движение персонала и работа горного мастера вне кабинета. Это и отдельный контур охраны труда, и часть общей цифровизации: рядом SAP, 1С, согласование ЛНА и кадровые процессы.</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Точный год старта и инициатор не названы. Уже есть подписание приказов и ознакомление в КЭДО. Причина, которая звучит: объём бумаги и ознакомлений (на разных предприятиях от 21 до 45 документов на человека), движение персонала и работа горного мастера вне кабинета. Это и отдельный контур охраны труда, и часть общей цифровизации: рядом SAP, 1С, согласование ЛНА и кадровые процессы.</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Единой даты старта нет. Письменно просили разрешить в пилоте электронное ознакомление с инструктажами вместо живой подписи и положительного ответа не получили. Параллельно все основные виды инструктажей уже фиксируют в своей системе, но без подписи. Отчёт о производственном контроле в электронном виде начали примерно в 2021 или 2022 году, точный год он не помнит. Причина: объём журналов, типография, время на подписи и непрозрачность по десяткам тысяч людей. Это решение службы охраны труда внутри более широкой кампании по сокращению лишней бумаги: предложения собирали у водителей и линейных руководителей. Полный текст — в файле Word этой компании.</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Электронного документооборота документов по охране труда как запущенного контура в записи нет. Сказано прямо, что с результатами работников электронно не знакомят: в кадровые системы отдают сведения о позициях, дальше коллеги организуют процесс. Договорный документооборот и доверенности были давно, ключи выданы широко. Кадровый контур жёстче. Когда и с какого документа охраны труда начали бы, не сказано, потому что этот перевод не описан. Причина, почему не идут в общую схему, — рабочие специальности не сидят онлайн, личные телефоны нельзя, внешний канал закрыт.</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Кадровые процессы на простой подписи идут давно. На усиленную неквалифицированную, по его оценке, перешли около двух лет назад, точность формулировки «второй год» в записи низкая. Обучение переводят в ЭДО с провайдером с 2023 года. Инструктажи под модель «одного ресурса» он считает для себя нереализуемыми, в том числе вводный. Наряды-допуски собираются сделать в этом году. Инициатор не назван. Причина движения — объём, в том числе колоссальный объём приёма, и желание не держать согласия только на бумаге. Причина, почему бумага ещё есть, — нестабильная позиция инспекции. Это часть общей цифровизации, не отдельный проект одной службы охраны труда.</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Отдельного старта ЭДО охраны труда нет. Зона документов есть, но она не стала, по смыслу фразы, полноценным электронным документооборотом; предыдущее название системы в расшифровке не восстановить. Кадровый ЭДО не внедрён и в ближайшие пару лет не планируется: группа переходит на другую версию платформы, название версии разобрать нельзя. Электронный допуск смотрели и бумагу не убрали, в историю «не дублируем» не пошли. Вводный инструктаж заносят в систему и печатают на живую подпись; ориентир по времени в записи — 2021 год, фраза шумная. Инициатор не назван. Причина осторожности — норму можно прочитать по-разному, плюс режим объекта и связь.</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="inlineStr">
+          <t>Точный год и инициатор не названы. Ознакомление с локальными актами уже идёт в КЭДО: блоки документов по должности загрузили и подвязали к приёму и переводу. Электронное подписание, по их словам, только стартует, целевая доля — 100%, потому что объектов много. Личные карточки в документооборот ещё не переведены целиком, этим занята проектная команда; звучит «блок в 1С», название модуля не разобрать. Отдельного решения «только служба охраны труда» или «вся цифровизация» они не формулируют: КЭДО уже общий контур приказов и ознакомления.</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>Дата старта одной фразой не названа. Ознакомление с локальными актами уже работает. Инструктажи начали переводить в ЭДО, исследователь уточняет, не в период ли её работы, прямой ответ в расшифровке тонет, дальше она говорит про аналитику. Почему ознакомление: меньше ходить и искать строку для подписи, можно поставить повтор раз в полгода или раз в три месяца и снизить риск, что человека не ознакомили. Это общий документооборот компании, не отдельная система службы охраны труда. Инициатор не назван.</t>
         </is>
@@ -705,9 +705,9 @@
           <t>Имени СЭД охраны труда нет. Есть система видеоинструктажа: вводный туда заносят и печатают. С 2025 года есть мобильное приложение и смартфоны, которые выдают на смену, не в личное пользование. Вход — учётная запись и пароль, для наряда-допуска носитель и пропуск информационная безопасность отклонила. Телефон пишет лог у себя и отдаёт его, когда появляется связь. Кадрового ЭДО нет. Старая система названа неразборчиво.</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Для приказов и ознакомления используют КЭДО. Руководитель утверждает документ, дальше его отправляют на ознакомление. Своя это разработка или купленная, спросили, ответ в записи не восстановить. Когда система появилась и для каких задач её брали сначала, не сказано. Стационарные компьютеры, по одной реплике, не выдают, подпись идёт через корпоративный контур; относить ли ноутбуки и корпоративный вайфай к словам компании, а не исследователей, по шуму нельзя, в ответ это не беру.</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -731,37 +731,37 @@
 Уточнения: Как принималось решение о выборе системы? Что было наиболее важным при выборе? Учитывались ли при выборе или внедрении системы особенности документов по охране труда? Какие именно?</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Итогового выбора системы под охрану труда ещё нет: в этом году рассчитывают открыть проект и сначала описать процессы верхнего уровня. Важное, что они сами называют: не вложить деньги и потом получить требование выгружать документы в госключ; ничего не хранить на внешних ресурсах; простой интерфейс, мало кнопок и полей. Особенности охраны труда в выборе звучат как мобильный персонал, карьер без связи, наряд, спецодежда, стажировка и наставник, а не как формальный чек-лист при закупке.</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Покупные системы не закрыли пакет, который они хотели завести в компанию, поэтому написали свою. Важными были прозрачность по всей массе работников, скорость, контроль сроков и возможность работать не только с компьютера. Особенности охраны труда закладывали сразу: инструктажи, наряд-допуск, предписания, производственный контроль, пожарный инструктаж, роли выдающего и допускающего. Отдельного протокола тендера он не пересказывал.</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Историю выбора СЭД под документы охраны труда не рассказали. По кадровому и договорному контуру важно другое: квалифицированная подпись, флешка-токен, свой удостоверяющий центр, а не госключ. Госключ он оценивает как «нам точно не надо». Особенности охраны труда на выбор системы не повлияли, потому что самого выбора под эти документы в записи нет: мешает периметр и то, что рабочие не у компьютера.</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Как выбирали систему, не рассказано. Наиболее важное, что он повторяет уже по итогам: не привязывать работодателя к одному ресурсу и не заставлять компанию, у которой система есть, жить в чужой. Особенности документов охраны труда при выборе в записи не фигурируют. Для наряда-допуска они сами делят процесс на наряд и допуск, это уже настройка, а не история закупки.</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Закупку отдельной СЭД под охрану труда не описывали. Выбор, который реально проговаривался, — с информационной безопасностью: для наряда оставили ввод пароля, без физической карты и без пропуска, хотя пароль можно передать. Корпоративный смартфон вместо личного — из-за данных и потому, что объект критический. Особенности охраны труда учтены так: подпись на месте, а не в кабинете, и работа без постоянного интернета. Когда появилась платформа, не сказано.</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>без ответа</t>
         </is>
@@ -807,9 +807,9 @@
           <t>Нет одной системы. Видеоинструктаж, приложение нарядов, бумажные журналы и сканы спецоценки живут рядом. Кадровый ЭДО документы охраны труда не покрывает. Интеграции «системы объезда» не достроены, фраза об этом обрывочная. Другие имена он не называет.</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Не все. Через КЭДО идут утверждение приказов и ознакомление с локальными актами. Личные карточки туда ещё не доведены. Инструктажи в КЭДО подписывают не всегда: «не успевают». Целевой инструктаж в разговоре отделяют от первичного и повторного. Спецоценка в эту же систему целиком не встаёт: опции приложить файл подписи эксперта к карте нет. Другие имена систем, кроме неясного блока 1С, не названы.</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -833,37 +833,37 @@
 Уточнения: Есть ли документы, которые вы хотели бы перевести в электронный формат, но система пока не позволяет этого сделать? Были ли документы, которые наоборот удалось перевести в ЭДО именно благодаря возможностям системы?</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Хотят, но система пока не даёт сквозной наряд: чтобы подтянулись заявка на спецодежду, срок стажировки и наставник. Сейчас это сбор в Excel, автоматизацией они это не считают. Личные карточки по охране труда проектная команда ещё не довела. По спецоценке в их контуре нет опции приложить файл подписи эксперта к той же карте, фраза об этом обрывочная. Удалось перевести ознакомление с локальными актами в КЭДО и на части предприятий выдавать электронное задание с идентификацией по карте.</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Хотят, но система пока не даёт сквозной наряд: чтобы подтянулись заявка на спецодежду, срок стажировки и наставник. Сейчас это сбор в Excel, автоматизацией они это не считают. По спецоценке в их контуре нет опции приложить файл подписи эксперта к той же карте, фраза об этом обрывочная. Удалось перевести ознакомление с локальными актами в КЭДО и на части предприятий выдавать электронное задание с идентификацией по карте.</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Технически готовы подписывать целевой инструктаж на наряде-допуске через УНЭП и пока этого не делают: ждут, можно ли так вообще, и уже много вложили. Спецоценку целиком в электронный вид не перевели: живая подпись остаётся, смена поставщика затормозила договорённость, что комиссия и работники подпишут УНЭП, а исполнитель подпишет у себя и передаст результат в портал. Госключ работникам хотят, это ещё проработка. Благодаря системе ушли от бумажного журнала трёхступенчатого контроля, собирают отчёт производственного контроля на любую дату, ведут предписания с закрытием, пожарный инструктаж подписывают УНЭП, протокол проверки знаний формируется автоматически.</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Хотели бы быстрее знать вредность и не ждать результат спецоценки до 12 месяцев: смежная служба уже требует назначенное рабочее место, класс условий сидит в мотивации, из-за лага они, по его словам, не дожидаются результата и потом пересчитывают прошедший год. В системах это не лечится, интеграции нет. Хотели бы, чтобы человек на входе прикладывал карту и видел, что ему нужно сделать, не выходя во внешнее решение. Что именно удалось перевести в ЭДО благодаря системе, по охране труда не названо. В кадровом контуре задание на согласие до работника доходит.</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Вводный инструктаж и вообще инструктажи в предложенной внешней модели он не видит, как реализовать: нужно ещё согласие на электронный оборот. Наряд-допуск хотят в этом году, наряд — полностью электронное согласование; что будет с допуском, фраза обрывается. Благодаря кабинету кадровые документы уже подписываются без госключа. Обучение ушло к провайдеру. Что система технически не умеет, кроме этой развилки, не сказано.</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Хотели бы не дублировать допуск, но не вошли в эту схему: смотрели опыт, где бумагу уже не ведут, и сами туда не пошли. Вводный можно было бы не печатать, но они печатают и подписывают от руки. Система видеоинструктажа как раз позволила заносить вводный и печатать его из системы, а не вести только журнал. Кадровые документы система не возьмёт ещё несколько лет из-за смены версии. Цифровизацию как тему он в разговоре про обучение готов отложить, хотя именно из-за неё встреча и собиралась.</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="inlineStr">
+          <t>Да. Личные карточки проект ещё не закрыл. По спецоценке систему нельзя заставить приложить к карте файл подписи эксперта, опции нет, это надо настраивать. Протокол проверки знаний они не собирают как один оригинал на весь южный дивизион. Благодаря КЭДО уже идёт ознакомление с набором документов по должности, и есть кнопка вернуть документ на подписание.</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>Да. Вводный инструктаж своим работникам не всегда проходит в тот же день, система не донастроена. В результат попадает тот, кто назначил инструктаж, а не руководитель, который его провёл, и сам руководитель в моменте не подписывает. Спецоценку и обучение нельзя честно считать электронными, пока внешняя организация не пришлёт документ, подписанный электронно, а не скан с живыми подписями. Благодаря системе получилось массовое ознакомление с отбором по человеку, должности и подразделению и повторные напоминания.</t>
         </is>
@@ -909,9 +909,9 @@
           <t>Помогает фиксация на месте: инструктор не кабинетный, отметка пишется в телефон и уходит в систему, когда аппарат попадает в сеть. Это для него надёжнее журнала, который потом уничтожают по сроку. Мешает отсутствие интернета и даже электричества на объекте, один объект Кольского филиала без нормальной связи, сменный телефон и пароль, который можно сказать другому, и то, что кадрового ЭДО не будет, пока группа меняет платформу. Юридически «можно и так, и по-другому» не даёт опереться на систему и выкинуть бумагу.</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>Помогает цепочка КЭДО: после подписи руководителя документ уходит на ознакомление, неподписанное можно вернуть на подписание. Мешает объём и география. В южном дивизионе одна комиссия на 50 городов, люди не успевают подписать в КЭДО, а дату в дату им нужно. По спецоценке удалённость мешает очному ознакомлению, а система не принимает файл подписи. Пример с тысячей пунктов выдачи они приводят сами: одну инструкцию нельзя размножить в тысячу оригиналов.</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -935,37 +935,37 @@
 Уточнения: Почему именно эти документы?</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Полного списка нет. В электронном виде ходят ознакомление с локальными актами и утверждение приказов и документов в КЭДО. На части предприятий есть электронное задание с идентификацией по карте. Почему эти: много людей, текучка и перестановки, без системы это не проконтролировать. Личные карточки по охране труда к полностью электронным они не относят.</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Полного списка нет. В электронном виде ходят ознакомление с локальными актами и утверждение приказов и документов в КЭДО. На части предприятий есть электронное задание с идентификацией по карте. Почему эти: много людей, текучка и перестановки, без системы это не проконтролировать.</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>Полностью без бумаги и без живой подписи он описывает журнал трёхступенчатого контроля и регистрацию, открытие и закрытие наряда-допуска: достаточно учётной записи и роли. Предписания производственного контроля и сбор отчёта тоже идут в системе, отчёт затем отдают в Ростехнадзор электронно вместе с экспертизами. Пожарный инструктаж и ознакомление с дефектной ведомостью экспертизы промышленной безопасности подписаны УНЭП. Почему так: пожарный инструктаж, по его словам, не попадает под ограничения приказа об обучении по охране труда, а трёхступенчатый контроль и регистрацию наряда они сознательно оставили на учётной записи. Полный текст — в файле Word этой компании.</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Таких документов по охране труда он не назвал. Прямо сказано, что электронно работников с этими результатами не знакомят. В электронном виде ходят сведения для кадровой системы и данные допуска подрядчиков, это не подписанный документ охраны труда.</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Полного списка документов охраны труда, которые только электронные, нет. Обучение переводят в ЭДО с 2023 года. Кадровые документы в личном кабинете электронные, это не охрана труда. Почему начали с них, он не объясняет отдельно: кадры были готовы раньше.</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>Полностью электронных документов охраны труда он не назвал. Вводный есть в системе и всё равно печатается на подпись. Наряд в приложении бумагу не заменил. Спецоценку подписывали в классическом виде и сканировали.</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J10" s="6" t="inlineStr">
+          <t>Полностью электронным они описывают ознакомление с локальными актами в КЭДО, блоками по должности. Почему эти: набор повторяется, а пунктов выдачи около тысячи, делать на каждый отдельный оригинал инструкции они не могут и не считают нужным. Инструктажи, протоколы и личные карточки к полностью электронным не относят.</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>Полностью электронным она описывает ознакомление с локальными актами: сообщение, вход, подпись в системе. Почему они: документы общие и цеховые, адресатов много, бумага здесь как раз лишняя. Инструктажи, спецоценка и обучение к полностью электронным не относятся, бумагу по ним дублируют.</t>
         </is>
@@ -988,7 +988,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Закрытого списка «только бумага» нет. Бумага остаётся там, где процесса в системе ещё нет: личные карточки, сквозной наряд, часть спецоценки. Отдельно — площадка без связи: перед выездом на карьер подписать негде, горный мастер не сидит в кабинете. Оригиналы по спецоценке люди по-прежнему просят. Причина в записи: нет устойчивой связи, нет готового процесса и жёсткая политика информационной безопасности.</t>
+          <t>Закрытого списка «только бумага» нет. Бумага остаётся там, где процесса в системе ещё нет: сквозной наряд и часть спецоценки. Отдельно — площадка без связи: перед выездом на карьер подписать негде, горный мастер не сидит в кабинете. Оригиналы по спецоценке люди по-прежнему просят. Причина в записи: нет устойчивой связи, нет готового процесса и жёсткая политика информационной безопасности.</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -1011,9 +1011,9 @@
           <t>На бумаге остаются подпись вводного, наряды-допуски и спецоценка. Обязательную форму наряда он выделяет только для одного вида работ, в расшифровке это звучит как правила при эксплуатации, точное имя правил не разобрать; остальные формы, по его словам, рекомендательные. Почему бумага: нет однозначного разрешения, первое лицо не взяло схему без дубля, связь на объекте не гарантирована.</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Закрытого списка нет. Инструкция по охране труда для сотрудника пункта выдачи одна на все точки, листа подписи в ней нет, листы ознакомления идут отдельно. Протокол проверки знаний физически гоняют копиями, пока не соберётся комиссия. Личные карточки в электронный оборот не доведены. Спецоценку в удалённых точках бумагой и копией карты они ещё обсуждают как действующее ограничение, а не как отменённый порядок.</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1037,37 +1037,37 @@
 Уточнения: Бывает ли, что полностью оформленный электронный документ всё равно распечатывается? Зачем? Кто принимает решение?</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Одновременно в двух видах прямо как регламент не описано. КЭДО умеет выгрузить документ на бумагу, если это нужно. По спецоценке обсуждали подпись эксперта и отдельное ознакомление работника со скан-копией карты; это описано как ограничение системы, а не как принятое правило «печатаем всегда». Кто решает печать, не сказано. Разговор про копии протоколов «южного дивизиона» в ответ не включён: по записи не отделить речь компании от примера собеседника.</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>Да. Семь видов инструктажей по охране труда, в том числе вводный, первичный, повторный и внеплановый, фиксируются в системе (дата, кто провёл, кому, тема), а подпись остаётся живой. Целевой инструктаж на работы повышенной опасности ведут электронно и печатают на живую подпись, эти подписи хранят 30 дней, как требуют по наряду-допуску. Протокол проверки знаний ещё дублируют и дубль отменяют. Спецоценку подгружают в систему и параллельно не ушли от живой подписи. Кто лично решает печать, не сказано: печать привязана к требованию закона, а не к выбору работника.</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>Прямо не сказано, что один и тот же готовый электронный документ ещё и печатают и кто это решает. Бумага и электронный контур существуют рядом: инспекция, по его словам, не даёт спокойно оставить только электрон, а часть процессов уже не пускает человека дальше без электронной подписи.</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>Да. Вводный заносят электронно и печатают на живую подпись. Наряд смотрели в электронном виде и дублируют бумагой. Спецоценка — живые подписи и скан. Кто утверждает печать, не сказано: для вводного печать встроена в порядок, для наряда они сознательно не перешли к чужому опыту без бумаги.</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J12" s="6" t="inlineStr">
+          <t>Да, для протокола. Оригинал один на южный дивизион, его копируют и пересылают по 50 городам, пока комиссия не соберёт подписи. Они прямо говорят, что так нарушают правило одного документа, и всё равно оригинал не собирают. Печать из системы как запасной путь звучит обрывочно: руководителю можно было бы сформировать запись, распечатать и подписать. Кто утверждает именно печать, не сказано.</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>Да, бумагу полностью дублируют, хотя ознакомление в системе есть. По спецоценке и обучению это прямо связано с тем, что электронный файл работника не заменяет подписи комиссии и эксперта. Печатается ли уже полностью подписанный электронный документ ещё раз и кто это решает, не сказано. Дубль описан как их текущее правило на переходный период, а не как разовая печать.</t>
         </is>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Да. Сквозной наряд со спецодеждой, стажировкой и наставником — пока Excel. Личные карточки не доведены. Инструктажи, ознакомление в поле и обучение они относят к процессам, которые надо переводить, но не хотят завязывать на внешний контур. Мешают отсутствие понятных правил, запрет выносить документы наружу, нет связи на карьере и несвязанные системы. Чтобы сдвинуться, им нужны правила до затрат, подпись внутри своей системы «нажал и подписал» и связь либо отдельный порядок для выезда.</t>
+          <t>Да. Сквозной наряд со спецодеждой, стажировкой и наставником — пока Excel. Инструктажи, ознакомление в поле и обучение они относят к процессам, которые надо переводить, но не хотят завязывать на внешний контур. Мешают отсутствие понятных правил, запрет выносить документы наружу, нет связи на карьере и несвязанные системы. Чтобы сдвинуться, им нужны правила до затрат, подпись внутри своей системы «нажал и подписал» и связь либо отдельный порядок для выезда.</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -1113,9 +1113,9 @@
           <t>Массовые инструктажи и наряд без бумажного дубля. Мешают неоднозначные разъяснения («можно и так, и иначе»), ответственность первого лица, отсутствие кадрового ЭДО на ближайшие годы, режим критической инфраструктуры и связь. Должно измениться правило: электронная фиксация достаточна, а не один из вариантов. Плюс устройство и канал, которые информационная безопасность пустит на объект.</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Да. Личные карточки: проект не закончен. Протокол: нельзя честно оставить один электронный документ, пока комиссия разъезжает по 50 городам и подписывает копии. Спецоценка: нет опции приложить файл подписи, а из-за удалённости с картой знакомят копией. Инструктаж на наряде-допуске они не ждут быстрым: если людям придётся ещё писать причины, в разговоре звучит, что этого скорее не сделают. Чтобы сдвинуться, нужна настройка системы под файл подписи и правило, которое не требует тысячу оригиналов и очный сбор комиссии.</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1139,37 +1139,37 @@
 Уточнения: Кто инициирует документ? Где он создаётся? Кто его заполняет? Кто проверяет? Кто подписывает? Кому передаётся? Где хранится? Кто имеет доступ? Что происходит, если в документе обнаруживается ошибка? Как оформляется исправление? Что происходит с предыдущей версией?</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Один документ от создания до хранения целиком не разбирали. Частично: приказ или утверждаемый документ подписывает руководитель в КЭДО, затем помощник отправляет его на ознакомление. Если человек не подписал в срок, документ аннулируется; есть возврат на повторное подписание. Выгрузить документ и подписи можно. По спецоценке карта эксперта с файлом подписи в систему не грузится, опции нет. Кто проверяет, кто имеет доступ и что происходит со старой версией при ошибке — не сказано.</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>Целиком один документ с исправлением ошибки и судьбой старой версии не разобрали. Наряд-допуск: выдающий заходит под своей учётной записью и только при нужной роли, допускающий подтверждает, производитель работ вписывает бригаду и темы инструктажа, затем лист печатают на живую подпись. УНЭП на этом шаге подготовлен и выключен. Предписание производственного контроля создаёт тот, кто выявил несоответствие, закрывает ответственный, оба под своими учётными записями, чужой логин передавать нельзя. Отчёт собирается на любую дату и уходит в Ростехнадзор с приложениями. Протокол проверки знаний формируется после практики и экзамена и рассылается на ознакомление. Полный текст — в файле Word этой компании.</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>Полный путь одного документа не разобран, кусок записи про наряд пропущен расшифровкой. Спецоценка: узкое место — подписи членов комиссии, обход занимает много времени; кто создаёт карту, где она хранится и как правят ошибку, не сказано. Наряд-допуск делят на наряд и допуск, наряд будет целиком в электронном согласовании. Кадровый документ в личном кабинете работник подписывает сам, иначе не двигается связанный процесс, пример — выдача машины.</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>Полной цепочки с проверкой, ошибкой и старой версией нет. Вводный: заносят в систему видеоинструктажа, печатают, подписывают от руки. Наряд: смартфон на смену, работник входит под своей учётной записью паролем, событие пишется логом в телефоне, время прикладывания или отметки хранится в аппарате и синхронизируется, когда телефон попадает в сеть станции или в город. Кто создаёт наряд и кто его проверяет, не разложено. Спецоценка подписывалась на бумаге и сканировалась. Где сервер и кто смотрит архив, не сказано.</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J14" s="6" t="inlineStr">
+          <t>Один документ целиком, с ошибкой и судьбой старой версии, не разобрали. Приказ: руководитель подписывает в КЭДО, затем документ уходит на ознакомление. Если работник не подписал, есть возврат на подписание. Модель «зашёл, значит подписал» они отвергли: разрешения не нашли. Протокол: дата проверки знаний может быть раньше, чем подписи членов комиссии; обсуждали, что подписи надо собрать заранее, примерно за неделю до конца срока обучения, иначе с даты в протоколе допуск уже спорный. По спецоценке работник может подписать одну карту, а эксперт подписывал весь отчёт; они хотят архив, где к нужной карте приложен файл подписи, и говорят, что такой опции нет. Полный текст — в файле Word этой компании.</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>Локальный акт: руководитель кадров или охрана труда загружает файл, выбирает фамилии, должности или подразделение, человеку приходит сообщение, он заходит и ставит подпись. Если молчит, она пишет ему сама или через линейного руководителя; руководители тоже опаздывают. Хранится в системе, на сервере компании, отдельный архив не делали. Доступ у работника по паролю, круглосуточно, с рабочего компьютера, телефона или из дома. Инструктаж: она назначает, система запоминает назначившего, а не того, кто провёл; подпись односторонняя, руководитель в моменте не подписывает. Что делают с ошибкой и со старой версией, не сказано.</t>
         </is>
@@ -1215,9 +1215,9 @@
           <t>Одинакового порядка нет. Вводный — рукописная подпись на листе из системы. Наряд в приложении — пароль учётной записи, отдельным видом электронной подписи он это не называет. Спецоценка — живая подпись и скан. Кадровой квалифицированной подписи у них нет, контур не внедрён.</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Нет. Утверждение приказа в КЭДО и ознакомление — разные шаги, второй идёт после первого. Ознакомление они не считают автоматическим фактом входа. Протокол живёт своей датой и поздними подписями комиссии. На вопрос про одну подпись на документе по спецоценке отвечают, что так и будут делать, но как именно выровняют вид подписи, не договаривают. Целевой инструктаж подписывает охрана труда, первичный и повторный заводит руководитель.</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1241,37 +1241,37 @@
 Уточнения: От чего зависит вид ЭП (кто и какие виды ЭП использует)?</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Матрицы «кто каким видом подписи подписывает» компания не проговорила. Сказано, что типы подписей в системе разные и простая подпись тоже есть. Старт электронной подписи они связывают с согласием работника, в том числе при трудоустройстве; дословно согласие не зачитано. Для процессов, где факт нужно доказать, документы во внешний контур уводить не хотят.</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>Вид зависит от того, считает ли компания действие подписью и что требует надзор или правило. Учётная запись — где они договорились внутри, что это фиксация роли, а не подпись. УНЭП — где надзор когда-то просил подтвердить ознакомление с экспертизой (сейчас, по его словам, уже не просит, но они оставили) и где пожарный инструктаж удалось вынести из-под ограничений обучения по охране труда. Для работников квалифицированную подпись он считает дорогой. Матрицы по должностям нет.</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>По охране труда зависимость вида подписи не задана. В кадрах вид зависит от того, зафиксирована ли бумажная форма актом: такие формы в КЭДО переводить сложно, остальное может идти простой подписью. Квалифицированный токен — у тех, кому выдали ключ и кто участвует в конкретном шаге. Рабочий персонал в эту схему не посажен.</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>От процесса. Внешнее подписание — квалифицированная подпись. Внутренние кадровые документы — подпись личного кабинета. Охрана труда на этот шаблон не посажена: комиссия спецоценки до сих пор самое долгое место, инструктажи не переведены. Кто из работников каким видом владеет, поимённо не сказано.</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>От процесса и от информационной безопасности, а не от матрицы документов. Для приложения наряда выбрали пароль, физический носитель исключили. Усиленную подпись для охраны труда он не описывает. Живая подпись остаётся там, где они не готовы отвечать за отказ от бумаги.</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J16" s="6" t="inlineStr">
+          <t>Матрицы нет. Вид зависит от шага. Ознакомление в КЭДО — отдельное действие работника, исследователь называет его простой подписью, компания это слово как термин не произносит. Подпись руководителя на утверждении в одном месте звучит как усиленная, фраза шумная, вид подписи дословно не фиксирую. Для протокола важен не вид носителя, а то, что подписи комиссии приходят позже даты протокола. Внешних подписантов спецоценки в ту же схему они пока не посадили.</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>От документа и от того, кто вне компании. Внутреннее ознакомление закрывает подпись входа в ЭДО. Где подписантов много и они внешние, вид подписи они пока не выровняли: живая подпись остаётся у комиссии и эксперта. Матрицы по должностям нет.</t>
         </is>
@@ -1292,7 +1292,7 @@
 Уточнения: Если используется ПЭП: в какой форме используется ПЭП (код из СМС или почты, логин и пароль от корпоративной системы, логин и пароль от Госуслуг, другое)?</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>без ответа</t>
         </is>
@@ -1302,12 +1302,12 @@
           <t>Как ПЭП они учётную запись не квалифицируют и форму ПЭП не описывают. Фактически человек входит в свою учётную запись, система пускает его только при нужной роли. Код из СМС, почта и логин Госуслуг не названы.</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>без ответа</t>
         </is>
@@ -1317,9 +1317,9 @@
           <t>Словом «ПЭП» он пароль не называет. Фактически для наряда это логин и пароль корпоративного приложения на сменном смартфоне. СМС, почта и Госуслуги не используются. Пароль можно передать другому, они это понимают и всё равно остановились на пароле.</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Код из СМС, почта и логин Госуслуг не названы. По тому, как показывают ознакомление, работник в корпоративном контуре нажимает, что ознакомлен, и на этом шаге формируется отметка. Это описание процесса, а не выбранная ими формулировка «у нас ПЭП такая-то».</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1343,37 +1343,37 @@
 Уточнения: Используете ли в качестве ЭП Госключ?</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>Госключ как штатный способ подписи документов по охране труда не описан. Позиция жёсткая: инструкции и документы охраны труда во внешние ресурсы не выкладывают, политика информационной безопасности это запрещает, часть сведений может быть коммерческой. Подписание в государственной системе означало бы отдать документы наружу. Продление электронной подписи через Госуслуги упоминается, это не то же самое, что подпись госключом. Фрагмент «подпись через КОТ» неразборчив.</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>В работе у работников госключа нет. Он говорит, что госключ хотят, и это пока проработка, не внедрение. Портал «Работа в России» в этой части разбирает исследователь: функций не хватает, документ откуда возьмётся и какой будет формы, непонятно. Ответ компании на это — нельзя навязать любое готовое решение, интеграция будет трудоёмкой.</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>Нет. Свой удостоверяющий центр есть, госключ он считает неподходящим: «нам точно не надо». Работник не будет подписывать документы госключом на том устройстве, которое стоит на площадке. Либо госключ, либо свой центр — развилка, которую он проговаривает, и компания остаётся при своём центре.</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>Для внутренних кадровых и, судя по контексту, охрано-трудовых документов госключ не используют. Им пользуются, когда зависают Госуслуги и нужно взаимодействие с Социальным фондом и другими государственными сервисами. Он считает эту подпись тоже личной. Упрощённая процедура госключа «у ребят» упомянута неразборчиво, как устроен допуск, не восстановить.</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>Нет. На вопрос про госключ на несменном личном устройстве он отвечает, что схема и так усложнённая: даже корпоративный смартфон дался тяжело, люди на смене меняются, личный телефон они не используют. Внедрения госключа нет.</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J18" s="5" t="inlineStr">
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>без ответа</t>
         </is>
@@ -1419,9 +1419,9 @@
           <t>Да. Пароль на общем телефоне можно передать, постоянной сети нет, поэтому подпись не онлайн, а отложенным логом, и он сам говорит, что отложенную передачу могут не принять. Пока это не признано, бумажный дубль не снимают. Отдельный пример, почему одной бумаги мало: при расследовании не нашли журнал инструктажа на рабочем месте, его уничтожили по сроку хранения. Это не сбой электронной подписи, но это причина не верить, что бумага сама по себе сохранит факт.</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Да. Люди не успевают подписать в КЭДО, а дата нужна день в день. Протокол одной даты и подписи комиссии другой ломают срок обучения. Разные виды подписи на одном документе они сами упирают в спецоценку: скан с живой подписью и электронная подпись работника вместе, по смыслу разговора, документ не собирается. Файл подписи эксперта система не принимает. Из-за этого удалённые точки остаются на копиях, а не на одном электронном оригинале.</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1445,37 +1445,37 @@
 Уточнения: С какими документами знакомятся электронно? Как работник получает документ? Как подтверждается ознакомление? Как фиксируются дата и время? Что происходит, если работник не ознакомился? Как организуется массовое ознакомление? Как работаете с персоналом, который не имеет постоянного доступа к компьютеру? Есть ли документы, с которыми вы не можете организовать полноценное электронное ознакомление, хотя хотели бы это сделать? Почему?</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>Электронно знакомят с локальными актами. Блоки документов по должности загружены в кадровый контур и поднимаются при приёме и переводе. Работнику приходит задача в КЭДО, он подписывает. Не подписал — напоминание каждый день, затем аннулирование; можно вернуть на подписание и можно отказаться, написав причину. Массовая рассылка идёт после подписи руководителя. Дата и время именно ознакомления отдельной фразой не названы, фиксируется срок и факт просрочки. Офисным выдают ноутбуки и корпоративную сеть, стационарные компьютеры — нет. Полный текст — в файле Word этой компании.</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Электронно знакомят с локальными актами. Работнику приходит задача в КЭДО, он подписывает. Не подписал — напоминание каждый день, затем аннулирование; можно вернуть на подписание и можно отказаться, написав причину. Массовая рассылка идёт после подписи руководителя. Дата и время именно ознакомления отдельной фразой не названы, фиксируется срок и факт просрочки. Для обязательной фиксации в поле устройства собираются закупать; личный телефон годится, чтобы посмотреть нормы и обучение в личном кабинете, но не как норма для обязательной подписи. Интерфейс должен быть простым. Полноценно не получается ознакомить там, где нет связи перед выездом на карьер. Полный текст — в файле Word этой компании.</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>Электронно доводят протокол проверки знаний, пожарный инструктаж и ознакомление с дефектной ведомостью. По инструктажам охраны труда в системе есть факт, но не подпись работника. Сообщение приходит на компьютер или в мобильное приложение, человек подтверждает под учётной записью либо подписывает УНЭП. Дата инструктажа фиксируется; про часы и минуты подписи отдельной фразы нет. Если срок устранения или контроля прошёл, система напоминает. Массово это закрывает более 35 тысяч человек. У кого нет смартфона, есть компьютерные классы: таких остались единицы, в основном возрастные с кнопочными телефонами. Дома пользоваться можно. Полный текст — в файле Word этой компании.</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>Электронного ознакомления работников с документами охраны труда нет: «электрон нет, мы не знакомы», в кадры уходят сведения. Как работник получил бы документ, как ставится время и что будет, если не ознакомился, для охраны труда не описано. Массовое ознакомление не организовано. Почты у рабочих нет, онлайн они не сидят, личные телефоны нельзя. Карта, которой человек отмечается на табло, — желаемая схема и практика, которую он видел у энергетиков и у подрядного пропуска, а не действующее ознакомление с инструкцией. Документы, которые хотели бы так знакомить, — результаты, завязанные на рабочее место и допуск, но внешнего решения им нельзя.</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>Как именно работник знакомится с документом охраны труда, не рассказано: ни канал, ни фиксация времени, ни последствия, если человек не открыл документ. Рабочему персоналу устройства, по обрывочной фразе, скорее не выдают; сам он корпоративным пользуется только для теста. Есть места, где интернета нет, при этом по восьми заводам в крупных городах связь в целом есть, противопоставление в записи смазано. Сопротивление переходу с рукописной подписи было выше, сейчас около одного процента. Часть не охрано-трудовых процессов просто не пускает дальше без электронной подписи. Полноценного электронного ознакомления с инструктажами нет.</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>С вводным знакомят через видеоинструктаж, подтверждение — подпись на распечатке. На месте отметка может лечь в телефон и уйти позже, когда аппарат в зоне связи; так он описывает и удалённую точку. Дата и время пишутся в лог телефона в момент отметки, на сервер попадают не сразу. Что будет, если человек не отметился, не сказано. Массовое ознакомление не запускали: «зачем мне это вводить», пока инструктаж как электронный процесс не принят. Компьютера у работника на объекте нет, вместо него сменный смартфон. Полноценно не ознакомить электронно те инструктажи, которые они не переводят, и любой факт на Кольском объекте, пока человек не дойдёт до связи.</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J20" s="6" t="inlineStr">
+          <t>Электронно знакомят с локальными актами по должности: блок уже загружен и поднимается при приёме и переводе. Человеку приходит документ в КЭДО, он отмечает ознакомление. Если не подписал, документ можно вернуть на подписание. Дата и время отдельной фразой не названы. Массово это один и тот же набор, а не тысяча разных оригиналов: инструкция для пункта выдачи одна на все точки, лист ознакомления отдельно, в инструкции нет места для подписи. Что будет, если человек так и не откроет документ, кроме возврата на подписание, не сказано. Про собственные телефоны спросили, разборчивого ответа нет. Полный текст — в файле Word этой компании.</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
         <is>
           <t>Электронно знакомят с локальными актами, в том числе отдельными для складов, не со всей компанией. Человеку приходит сообщение зайти и ознакомиться, он ставит подпись. Время подписи фиксируется. Если не ознакомился, она напоминает лично или через руководителя, плюс можно настроить повтор пакета раз в три или шесть месяцев. Массово — выбором категории, должности или подразделения. Линейный персонал чаще подписывает с личного телефона. Это не обязанность: есть рабочий компьютер с паролем, можно из дома, круглосуточно, положение об ЭДО есть, запрета личного телефона нет, аналитики «кто с какого устройства» нет. Полный текст — в файле Word этой компании.</t>
         </is>
@@ -1521,9 +1521,9 @@
           <t>Да. Письмо с разъяснением, по его пересказу, звучало как «можно и так, и по-другому», поэтому на электронный допуск без бумаги они не опёрлись. В правилах по охране труда формулировка про оборот похожая, но этого им мало. Срок хранения журнала инструктажа менялся: он рассказывает про журнал 2008–2009 годов, который при десятилетнем сроке уничтожили, и при несчастном случае подтвердить инструктаж двадцатилетней давности было нечем. Требование хранить бумагу долго не помогло. Про один вид подписи на документе спецоценки он знает, свою действующую схему скана из-за этого порочной прямо не называет.</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Да. Модель «открыл документ — уже ознакомился» отвергли: запрета не нашли, но и разрешения тоже, поэтому от схемы отказались. Протокол по требованиям должен быть одним документом, с программой, датой и тем, кому проведено; копии они всё равно возят по дивизиону и говорят, что так нарушают. Риск считают низким, пока документ не запросили. Отдельно обрывается реплика, что Настю или коллегу штрафовали из-за члена комиссии; за что именно, не разобрать. Где норма была неясна, они выбирают более осторожный вариант, а не отказ от КЭДО.</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1547,37 +1547,37 @@
 Уточнения: Какие из них, на ваш взгляд, необходимо изменить или уточнить?</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>Сильнее всего, по их словам, мешает отсутствие правил и риск, что после внедрения обяжут внешний инструмент, в первую очередь госключ и выгрузку документов наружу. Второй ограничитель — связь и мобильный персонал: страну нормальной связью они не покроют, а горный мастер не должен сидеть в кабинете. Уточнить они хотят не статью закона, а развилку: подпись внутри своей системы, без лишних действий и без раскрытия инструкций. Пока этого нет, коммерческий собственник, по их оценке, скорее наймёт людей, чем заплатит за то, чего закон прямо не требует.</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>Сильнее всего держат запрет и неясность электронной подписи инструктажей и то, что без обязательного требования они не идут в дорогой внешний контур. Отдельно мешает отсутствие единого описания: электронный наряд, журнал регистрации, пожарные инструктажи и обычные инструктажи описаны кусками в разных документах, общий стандарт только собираются сделать. Что изменить: чтобы электронную фиксацию инструктажа можно было не дублировать бумагой и чтобы это не было приклеено к одному порталу, в котором не хватает функций. Конкретных пунктов актов он не перечислял.</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>Сильнее всего ограничивают не одна цитата из приказа, а связка: человек не в сети, личные устройства нельзя, бумажная форма части документов, спецоценка только через рабочее место и долгий лаг. Менять, по его позиции, нужно не в сторону единого портала. Если государству нужен факт, компания готова отдавать сведения из своей системы, как уже отдаёт кадровую отчётность. Навязанный канал и госключ он просит не вводить: виды подписей и так заданы законом об электронной подписи. Конкретные пункты для правки не продиктованы.</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>Сильнее всего ограничивает идея одного обязательного ресурса и цена интеграции для компании, где система уже есть, плюс неясность, примет ли инспекция электронный документ. Изменить он предлагает сам принцип: разрешить, как в кадровом ЭДО, а не назначить площадку. Для малого бизнеса государственный ресурс без своей платформы он считает нормальным. Что расписать в норме по шагам, не говорит: сотрудники привыкли к одной экосистеме, второй контур будет лишним.</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>Ограничивает неясность: электронный оборот в правилах вроде допускается и одновременно официально можно оставить любой вариант. Второй ограничитель — бумажный журнал как единственное доказательство, которое ещё и уничтожается по сроку. Уточнить нужно, что электронной фиксации достаточно. Текст правки он не предлагает. Запрет инструктажей в записи проговаривает в основном исследователь, компания отвечает примером вводного, который всё равно печатают.</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J22" s="6" t="inlineStr">
+          <t>Сильнее всего мешают правило одного документа и одной вида подписи там, где люди и комиссия разъеханы: 50 городов южного дивизиона и около тысячи пунктов выдачи. Второе — система не умеет приложить файл подписи к карте спецоценки. Что изменить, они списком не говорят. По смыслу реплик им нужно ознакомление без тысячи оригиналов и протокол, который не надо физически собирать. Пункты актов не назывались.</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
         <is>
           <t>Ограничивают правило одной вида подписи на документ и невозможность оставить инструктаж только в электронном виде. Изменить ей нужно первое, чтобы дубль бумаги по инструктажу после переходного периода можно было снять, и практику, при которой внешняя организация отдаёт файл с подписью, а не скан. Пункты актов она не называет. Что не стоит регулировать слишком подробно, не обсуждала.</t>
         </is>
@@ -1623,9 +1623,9 @@
           <t>Эффект от перевода документов охраны труда не считали: перевода нет. Отдельно и долго говорили про убытки от происшествий и культуру безопасности, эти проценты выручки и данные для Минэнерго к ЭДО не относятся, в ответ их не переношу. Единственный практический урок про документы — бумажный журнал не спас при расследовании, потому что был уничтожен. Экономию времени на подписи он не называл.</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Расчёта эффекта нет. Качественно они описывают не «стало быстрее на столько-то», а почему бумага не масштабируется: одну инструкцию нельзя выпустить тысячей оригиналов, комиссию по 50 городам не собрать на один лист, ознакомление по должности уже уходит в КЭДО при приёме и переводе. Ошибки, поиск и хранение цифрами не оценены. Доля электронного подписания, по их словам, только начинается, цель — 100%.</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1649,37 +1649,37 @@
 Уточнения: Почему?</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J24" s="5" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="inlineStr">
         <is>
           <t>без ответа</t>
         </is>
@@ -1700,7 +1700,7 @@
 Уточнения: Почему?</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>без ответа</t>
         </is>
@@ -1710,22 +1710,22 @@
           <t>Один документ лучшим он не назвал. Самым большим эффектом назвал сокращение времени на наряд-допуск и на служебные письма и поручения, отдельно — отказ от закупки бумажных журналов. Прозрачность инструктажей по десяткам тысяч человек для него тоже главный практический результат, хотя подпись там ещё бумажная.</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
         <is>
           <t>без ответа</t>
         </is>
@@ -1751,37 +1751,37 @@
 Уточнения: Какая проблема сегодня сильнее всего ограничивает дальнейший переход к электронному документообороту?</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>Самое сложное для них — двигаться без правил и не потратить бюджет на схему, которую потом заменят госключом или внешним порталом. Рядом: информационная безопасность не пускает документы наружу, на карьере нет связи, системы охраны труда не связаны между собой, а в TESSA работник теряется. Дальнейший переход сильнее всего держит связка «нет нормы + нельзя вынести документ наружу + человек не у компьютера».</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>Сложнее всего подпись и принятие её людьми: без большой разъяснительной кампании работники расходятся в понимании, зачем это. Дальше переход ограничивают неясность по инструктажам и нарядам-допускам, обрывы связи и то, что дорогое внешнее окно без отмены параллельных обязанностей они включать не будут. Хранение многолетних бумажных журналов как раз было причиной уйти в цифру, а не текущей проблемой системы.</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>Самое сложное — производственный персонал, который не находится в сети, при закрытом периметре: личные телефоны нельзя, где-то нет даже обычной телефонной связи, только внутренняя, на удалённой площадке программа еле открывается. Второй слой — спецоценка и кадры не стыкуются, системы самописные и почти не дорабатываются, а новое внедрение сейчас упирается в деньги и людей: раньше на развитие было легче. Дальнейший ЭДО охраны труда сильнее всего держит именно отсутствие постоянного цифрового доступа у рабочих плюс запрет выйти во внешний сервис.</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>Самое тяжёлое в охране труда на сегодня — собрать подписи комиссии по спецоценке. Дальше переход ограничивают один внешний ресурс и дорогая интеграция, устройства не у всех рабочих и остаточное нежелание переходить на электронную подпись, около одного процента. Инструктажи он прямо называет тем, что они не реализуют.</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="H26" s="5" t="inlineStr">
         <is>
           <t>Самое сложное — решиться убрать бумагу без однозначной нормы и без решения первого лица. Дальше мешают объект критической инфраструктуры, дыры связи, сменный телефон и то, что кадровый ЭДО появится нескоро из-за смены платформы. Сильнее всего дальнейший переход держит связка «норму можно прочитать трояко» и «связи на объекте нет».</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J26" s="6" t="inlineStr">
+          <t>Самое тяжёлое — собрать подпись там, где людей много и они не в одном городе: пункты выдачи, южный дивизион, комиссия, которая не успевает подписать протокол в КЭДО к нужной дате. Рядом система, в которой нет опции для файла подписи по спецоценке, и личные карточки, которые проект ещё не довёл. Дальше переход держит именно это, а не отсутствие самого КЭДО: ознакомление с актами уже электронное.</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
         <is>
           <t>Сложно на старте настроить систему и научить людей, куда нажимать. Дальше переход держат инструктажи — не фиксируется реальный руководитель и не всегда выходит день в день — и связка подписей по спецоценке и обучению. Пока это не закрыто, они дублируют бумагу и не считают переход законченным.</t>
         </is>
@@ -1827,9 +1827,9 @@
           <t>Полезно прямое правило, что результат инструктажа, зафиксированный электронно, достаточен, без формулы «можно и так, и иначе». Слишком подробно задавать носитель не стоит: у них уже работает локальный лог и поздняя синхронизация, и именно это проходит на объекте без интернета. Госключ и личное устройство он считает лишним усложнением. Это вывод из его рассказа, не список поправок.</t>
         </is>
       </c>
-      <c r="I27" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>Полезным для них было бы признать электронное ознакомление и один протокол без обязанности возить бумажный оригинал по десяткам городов и без тысяча копий инструкции. Слишком подробно задавать носитель они не просят. Это сборка из того, на что они жалуются, а не продиктованный текст поправок. Госключ и портал в их репликах как просьба не звучат.</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -1853,37 +1853,37 @@
 Уточнения: Если считает необходимым: что именно сегодня делает бумажное оформление неудобным или избыточным?</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>Да, для них это нужный перевод. Инструктажи, ознакомление и обучение названы процессами, где много людей, текучка и перестановки, и без системы это не контролировать. Бумага неудобна объёмом: 21–45 документов на человека, подписи, горный мастер не должен возвращаться в кабинет, перед выездом на карьер подписать часто негде.</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>Для них это уже необходимость: все основные инструктажи ведут электронно и упираются только в подпись. Бумага избыточна как второй контур: живая роспись, хранение 30 дней по целевому, контроль десятков тысяч людей и журналы, от которых они в других процедурах уже отказались.</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
         <is>
           <t>Саму возможность он приветствует: изменение «очень обрадовало». Бумагу при этом неудобной по шагам он не разбирает. Сразу оговаривается, что вводный инструктаж и соседние процедуры они у себя не реализуют, если вместе с разрешением придут согласие на электронный оборот и один внешний ресурс.</t>
         </is>
       </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>Однозначного «необходимо» нет. Вводный они уже ведут в системе и всё равно подписывают на бумаге. Массово переводить остальные не начинают. Неудобство бумаги показано на уничтоженном журнале и на том, что инструктор должен зафиксировать факт на месте, а не в кабинете. При этом он спрашивает, зачем вводить то, что пока не даёт простой замены.</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J28" s="6" t="inlineStr">
+          <t>Для объёма, который они описывают, бумага уже не работает: тысяча пунктов выдачи и одна инструкция, 50 городов и одна комиссия. Инструктажи при этом в КЭДО закрыты не до конца, люди не успевают подписать. Бумагу неудобной они показывают на копиях протокола и на невозможности сделать тысячу оригиналов, а не на пошаговом разборе журнала.</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
         <is>
           <t>Для них это уже нужная возможность: инструктажи в ЭДО внедряют и при снятии ограничения хотят пользоваться этим полностью. Бумажный дубль она не защищает, он временный. Что именно избыточно в бумажном листе, по шагам не разбирает: выигрыш описывает на ознакомлении — не ходить, не ловить подпись, видеть срок.</t>
         </is>
@@ -1904,17 +1904,17 @@
 Уточнения: Если не считает необходимым: почему, на ваш взгляд, электронное оформление результатов инструктажей не даст существенного эффекта?</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>без ответа</t>
         </is>
@@ -1929,12 +1929,12 @@
           <t>Существенного эффекта он пока не ждёт. Цифровизацию в ряду других задач готов отодвинуть. Пока норму читают по-разному, кадрового ЭДО нет, а связь на объекте не гарантирована, электронная форма не отменяет бумагу и добавляет спор, примут ли отложенную отправку лога. Поэтому вводный они не оставляют только в системе.</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J29" s="5" t="inlineStr">
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="inlineStr">
         <is>
           <t>без ответа</t>
         </is>
@@ -1955,37 +1955,37 @@
 Уточнения: Кто вносит сведения в СЭД? Где должен храниться результат? Кто должен иметь доступ?</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>Цельный алгоритм они не продиктовали. Из того, как описывают желаемую работу: человек на месте нажимает понятную кнопку и подписывает в своей системе, без выгрузки в другую; для обязательной фиксации компании нужно выданное устройство, для просмотра сведений хватает личного кабинета; результат лежит у них, а не на внешнем ресурсе; неподписавших видно фильтром. Кто именно вносит результат инструктажа, где строка хранения и кто имеет доступ, по ролям не разложено. Для карьера без связи такого алгоритма у них пока нет.</t>
         </is>
       </c>
-      <c r="E30" s="6" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>Отдельный «идеальный» сценарий он не рассказывал, он описывает уже собранный. Обычный инструктаж: в системе дата, кто провёл, кому и какая тема, не хватает только признанной подписи. Целевой: выдающий и допускающий действуют под учётной записью и ролью, производитель вносит бригаду и темы, подпись УНЭП вместо печати уже подготовлена. Результат хранится в их системе, доступ есть у охраны труда по всей компании и у роли на телефоне. Кто имеет право смотреть при проверке и как исправлять ошибку, не сказано.</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
         <is>
           <t>Готового идеала нет, есть их контур. Отметка на месте, в сменном смартфоне, под паролем работника. Время пишется в телефон сразу, в систему компании попадает, когда аппарат видит сеть станции или возвращается в зону связи. Кто вносит текст инструктажа, не сказано. Хранение сначала в телефоне, потом у них. Кто смотрит запись при проверке, не названо. Бумагу этот контур пока не заменяет.</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J30" s="6" t="inlineStr">
+          <t>Цельный алгоритм не продиктовали. Из обрывков: руководитель заводит первичный и повторный инструктаж, целевой подписывает охрана труда; система должна напомнить; запись можно вернуть на подписание, если человек не подписал; для наряда-допуска есть опасение, что писать причины никто не будет. Где хранится результат и кто его смотрит, не сказано. Для дивизиона у них сейчас не этот алгоритм, а один оригинал и копии, пока комиссия не соберётся.</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
         <is>
           <t>Цельного алгоритма она не предложила. По дырам текущей схемы ей нужно другое: инструктаж проводится в тот же день, в системе остаётся тот, кто реально провёл, а не только тот, кто назначил, работник подписывает результат, запись лежит в той же системе. Кто имеет доступ при проверке и кто вносит текст, если это не сам работник, не сказано. Это реконструкция из её претензий к системе, не отдельный проект.</t>
         </is>
@@ -2031,12 +2031,12 @@
           <t>Отдельной оценки портала «Работа в России» нет. Близко к модели он говорит про отложенную выгрузку: факт фиксируется без интернета и уходит позже, а такой поздний обмен могут не принять. Госключ на сменном телефоне для него слишком сложен. Пользу единого портала он не назвал. Проблемы, которые у него уже есть и которые модель повторит: нет интернета, объект закрытый, устройство не личное и не постоянное, люди территориально на станциях, в том числе на Кольском филиале.</t>
         </is>
       </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J31" s="5" t="inlineStr">
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
         <is>
           <t>без ответа</t>
         </is>
@@ -2057,37 +2057,37 @@
 Уточнения: Для каких категорий работников это может стать проблемой? Есть ли у вас работники, для которых такой способ идентификации будет затруднителен? Что делать, если работник не может или не хочет воспользоваться таким способом идентификации?</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>Прямо про ЕСИА не говорили. Обязательную фиксацию они не переносят на личный телефон: для неё планируют закупать устройства, а личный кабинет на своём телефоне — чтобы смотреть нормы и обучение. Трудные категории в их рассказе — люди на карьере и разъездной персонал без связи, плюс работники, которым нужен интерфейс из минимума кнопок. Что делать, если человек откажется от ЕСИА, не сказано. В КЭДО отказ от подписи с комментарием уже есть, но это другая система.</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>Про ЕСИА не говорили. Идентификация сейчас — своя учётная запись, на части задач телефон. Затруднительно это единицам с кнопочными телефонами, в основном возрастным, кто не хочет учиться: для них сделаны компьютерные классы, дома в приложении работать можно. Что делать при отказе именно от ЕСИА, не обсуждалось.</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="F32" s="5" t="inlineStr">
         <is>
           <t>Про ЕСИА прямо не говорили. Идентификация, которую они готовы обсуждать, — карта или токен внутри периметра, не личный телефон и не внешний сервис. Затруднительно это будет рабочим специальностям: почты нет, в онлайне они не сидят, личный телефон запрещён, на смену в других компаниях, по его примеру, выдают общее устройство. Что делать при отказе от ЕСИА, не сказано. Свой вариант — отметиться картой на месте и не выходить наружу.</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="H32" s="6" t="inlineStr">
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
         <is>
           <t>Про ЕСИА не говорили. Сейчас работник вводит пароль в корпоративном приложении на телефоне, который выдан на смену. Пароль можно сообщить другому, это принятый компромисс с информационной безопасностью. Личный телефон не используют, даже корпоративный смартфон внедряли с сопротивлением. Категория, которой будет трудно, — смена на объекте без связи и без личного устройства. Замены ЕСИА он не предлагал.</t>
         </is>
       </c>
-      <c r="I32" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J32" s="5" t="inlineStr">
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="inlineStr">
         <is>
           <t>без ответа</t>
         </is>
@@ -2133,12 +2133,12 @@
           <t>Связки с порталом нет. Кадровой СЭД, с которой портал мог бы обмениваться, в ближайшие годы не будет, группа меняет версию платформы. Запись они видят у себя после синхронизации телефона. Нужна ли отдельная копия, прямо не сказано: фактически она сначала лежит в телефоне, затем в их контуре. Автоматическую передачу на «Работу в России» не обсуждали.</t>
         </is>
       </c>
-      <c r="I33" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J33" s="5" t="inlineStr">
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
         <is>
           <t>без ответа</t>
         </is>
@@ -2158,37 +2158,37 @@
           <t>Если бы вам поручили сформулировать требования к будущей системе электронного оформления результатов инструктажей, какие три требования вы бы поставили на первое место?</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>Тремя пунктами не формулировали. Из разных реплик складываются такие условия: подпись внутри своей системы, без выгрузки и без госключа; минимум действий для работника, в том числе в поле; устойчивая связь либо понятный порядок для карьера и устройство, которое переживёт площадку. Это сборка, не дословный ответ на «назовите три требования».</t>
         </is>
       </c>
-      <c r="E34" s="6" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>Тремя требованиями не назвал. По тому, что уже сделано и чего не хватает, для него критичны признанная подпись там, где система готова (УНЭП на инструктаже и наряде), работа с учётной записи и с телефона без отдельного ключа на каждого и отсутствие второго обязательного контура — бумаги или внешнего портала. Это сборка из его описания, не список, который он продиктовал.</t>
         </is>
       </c>
-      <c r="F34" s="6" t="inlineStr">
+      <c r="F34" s="5" t="inlineStr">
         <is>
           <t>Тремя требованиями не назвал. По повторяющимся репликам для него важны: данные уходят из своей системы, а процесс на портал не переезжает; идентификация внутри периметра, без личного телефона; остаётся их удостоверяющий центр и токен, а не госключ. Это сборка, не продиктованный список.</t>
         </is>
       </c>
-      <c r="G34" s="6" t="inlineStr">
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>Тремя требованиями не назвал. По его комментарию к проекту на первом месте разрешение в логике кадрового ЭДО без обязательного единого ресурса, подпись в той системе, где люди уже работают, и интеграция, которая не стоит дороже самого перевода. Для малого бизнеса он готов оставить простой государственный вариант. Это сборка из комментария, не список из трёх пунктов.</t>
         </is>
       </c>
-      <c r="H34" s="6" t="inlineStr">
+      <c r="H34" s="5" t="inlineStr">
         <is>
           <t>Тремя требованиями не назвал. По собранному ими контуру на первом месте работа без постоянного интернета, идентификация, которую информационная безопасность пускает на сменное устройство, и правовое признание локального лога, чтобы бумагу можно было не дублировать. Это сборка, не его список.</t>
         </is>
       </c>
-      <c r="I34" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J34" s="6" t="inlineStr">
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
         <is>
           <t>Тремя требованиями она не назвала. По тому, что уже заставила систему делать и чего не хватает, для неё важны фиксация времени и факта подписи, в результате должен стоять реальный инструктор, а не только назначивший, и подпись с телефона или компьютера в той же системе, без отдельного хранилища. Это сборка, не её список.</t>
         </is>
@@ -2208,37 +2208,37 @@
           <t>Если бы вам нужно было дать один совет организации, которая только начинает переводить документы по охране труда в электронную форму, что бы вы посоветовали?</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="H35" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="I35" s="5" t="inlineStr">
-        <is>
-          <t>без ответа</t>
-        </is>
-      </c>
-      <c r="J35" s="5" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J35" s="6" t="inlineStr">
         <is>
           <t>без ответа</t>
         </is>

</xml_diff>

<commit_message>
Add a respondents-only sheet to the EDO interview workbook.
The second sheet keeps the 33 questions and the seven company columns, and drops personal names and interviewer-only figures from the cells.

Co-authored-by: lysakalenushka-hash <lysakalenushka-hash@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/транскрипции/Ответы по вопросам/Сводная по интервью ЭДО.xlsx
+++ b/транскрипции/Ответы по вопросам/Сводная по интервью ЭДО.xlsx
@@ -8,10 +8,13 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводная" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Только респонденты" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Сводная'!$A$2:$J$35</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Сводная'!$1:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Только респонденты'!$A$2:$J$35</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Только респонденты'!$1:$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2260,4 +2263,1783 @@
     <firstFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:J35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ответы компаний</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Блок</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Вопрос</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Ареал</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Металлоинвест</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Газпром нефть</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Балтика</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>ТГК-1</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>КУПИШУЗ (Ламода)</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>МЭЛОН ФЭШН ГРУП</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="210" customHeight="1">
+      <c r="A3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Блок 1. Роль респондента</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Расскажите, пожалуйста, о вашей роли в работе с документами по охране труда и ЭДО.
+Уточнения: За какие документы или направления вы отвечаете? Насколько участвуете в принятии решений по ЭДО? Участвовали ли во внедрении СЭД? С какими подразделениями взаимодействуете?</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Собеседник и коллеги со стороны охраны труда показывают, как на предприятиях устроены ознакомление, подписание и учёт, и обсуждают выбор системы. Личный перечень документов и формальное участие во внедрении конкретной СЭД в записи не названы: компания на этапе выбора системы и описания процессов верхнего уровня. В разговоре рядом информационная безопасность, площадки и горные мастера, а также внешние контуры обучения и спецоценки.</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Собеседник ведёт электронный контур охраны труда и промышленной безопасности по компании и сам давно занимается подписью. В системе больше 35 тысяч работников. Решения по тому, что оставить на бумаге, а что вести учётной записью или УНЭП, принимались у них, в том числе после отказа рынка закрыть нужный пакет. Рядом линейные руководители, работники, административный персонал, Ростехнадзор, учебный контур и организация, которая проводит спецоценку.</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Собеседник говорит со стороны охраны труда, но кадровый электронный документооборот относит к другим коллегам: эффект от отпусков и командировок — «не мой функционал». Его зона в записи — спецоценка, медосмотры, передача сведений в кадровые системы и ограничения для производственного персонала. В принятии решений по ЭДО охраны труда он описывает скорее рамку, чем внедрённый проект: системы функциональные, в основном самописные, интеграция не достроена. Рядом кадры, медицина, информационная безопасность, организация, которая делает спецоценку, и подрядчики на месторождениях.</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Собеседник говорит и про охрану труда, и про общий электронный контур: спецоценка, обучение, наряды-допуски, согласия, выдача машины. Насколько именно он утверждает выбор СЭД, не сказано. Кадры давно ведут свои процессы отдельно. Площадок в разговоре восемь заводов в крупных городах. Внешние подписи управленческих документов и провайдер обучения — отдельные контуры.</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Собеседник ведёт охрану труда по электростанциям и филиалам и говорит от первого лица про мобильное приложение, наряды-допуски и решение не отказываться от бумаги. В выборе «уйти с бумаги целиком» ключ, по его словам, у первого лица: надо принять ответственность. С информационной безопасностью он согласовывал вход в приложение. Учебный центр, филиалы, в том числе Кольский, и подрядчики в записи есть. Кадрового ЭДО у них нет, и это не его внедрение.</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Собеседник говорит со стороны охраны труда. Зона в разговоре — инструкции для пунктов выдачи, протоколы проверки знаний, ознакомление в КЭДО и личные карточки по охране труда. Насколько собеседник выбирал систему, не сказано. Рядом проектная команда по карточкам, кадры (блоки документов при приёме и переводе), руководители, которые заводят первичный и повторный инструктаж, и кладовщики: объектов много, фраза про кладовщика обрывается.</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>Собеседник — специалист по охране труда. Общие локальные акты в систему загружают двое: руководитель кадров и ответственный за группу охраны труда. Она сама кладёт документы подразделения, пример — склады, и выбирает, кому направить: по фамилии, должности или подразделению. Положение об электронном документообороте в компании есть. Архитектуру СЭД она не выбирала. Линейных руководителей подключает, когда люди не знакомятся вовремя. Для отчёта называет порядок численности тех, кто пользуется ЭДО: 9 тысяч.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="238" customHeight="1">
+      <c r="A4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Блок 2. Как в организации появился ЭДО по ОТ</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Расскажите, пожалуйста, как в вашей организации началось применение электронного документооборота в отношении документов по охране труда.
+Уточнения: Когда это началось? С каких документов начали? Почему начали именно с них? Кто выступил инициатором? Что стало причиной внедрения? Было ли это отдельное решение службы ОТ или часть общей цифровизации организации?</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Точный год старта и инициатор не названы. Уже есть подписание приказов и ознакомление в КЭДО. Причина, которая звучит: объём бумаги и ознакомлений (на разных предприятиях от 21 до 45 документов на человека), движение персонала и работа горного мастера вне кабинета. Это и отдельный контур охраны труда, и часть общей цифровизации: рядом SAP, 1С, согласование ЛНА и кадровые процессы.</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Единой даты старта нет. Письменно просили разрешить в пилоте электронное ознакомление с инструктажами вместо живой подписи и положительного ответа не получили. Параллельно все основные виды инструктажей уже фиксируют в своей системе, но без подписи. Отчёт о производственном контроле в электронном виде начали примерно в 2021 или 2022 году, точный год он не помнит. Причина: объём журналов, типография, время на подписи и непрозрачность по десяткам тысяч людей. Это решение службы охраны труда внутри более широкой кампании по сокращению лишней бумаги: предложения собирали у водителей и линейных руководителей. Полный текст — в файле Word этой компании.</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Электронного документооборота документов по охране труда как запущенного контура в записи нет. Сказано прямо, что с результатами работников электронно не знакомят: в кадровые системы отдают сведения о позициях, дальше коллеги организуют процесс. Договорный документооборот и доверенности были давно, ключи выданы широко. Кадровый контур жёстче. Когда и с какого документа охраны труда начали бы, не сказано, потому что этот перевод не описан. Причина, почему не идут в общую схему, — рабочие специальности не сидят онлайн, личные телефоны нельзя, внешний канал закрыт.</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Кадровые процессы на простой подписи идут давно. На усиленную неквалифицированную, по его оценке, перешли около двух лет назад, точность формулировки «второй год» в записи низкая. Обучение переводят в ЭДО с провайдером с 2023 года. Инструктажи под модель «одного ресурса» он считает для себя нереализуемыми, в том числе вводный. Наряды-допуски собираются сделать в этом году. Инициатор не назван. Причина движения — объём, в том числе колоссальный объём приёма, и желание не держать согласия только на бумаге. Причина, почему бумага ещё есть, — нестабильная позиция инспекции. Это часть общей цифровизации, не отдельный проект одной службы охраны труда.</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Отдельного старта ЭДО охраны труда нет. Зона документов есть, но она не стала, по смыслу фразы, полноценным электронным документооборотом; предыдущее название системы в расшифровке не восстановить. Кадровый ЭДО не внедрён и в ближайшие пару лет не планируется: группа переходит на другую версию платформы, название версии разобрать нельзя. Электронный допуск смотрели и бумагу не убрали, в историю «не дублируем» не пошли. Вводный инструктаж заносят в систему и печатают на живую подпись; ориентир по времени в записи — 2021 год, фраза шумная. Инициатор не назван. Причина осторожности — норму можно прочитать по-разному, плюс режим объекта и связь.</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Точный год и инициатор не названы. Ознакомление с локальными актами уже идёт в КЭДО: блоки документов по должности загрузили и подвязали к приёму и переводу. Электронное подписание, по их словам, только стартует, целевая доля — 100%, потому что объектов много. Личные карточки в документооборот ещё не переведены целиком, этим занята проектная команда; звучит «блок в 1С», название модуля не разобрать. Отдельного решения «только служба охраны труда» или «вся цифровизация» они не формулируют: КЭДО уже общий контур приказов и ознакомления.</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Дата старта одной фразой не названа. Ознакомление с локальными актами уже работает. Инструктажи начали переводить в ЭДО. Почему ознакомление: меньше ходить и искать строку для подписи, можно поставить повтор раз в полгода или раз в три месяца и снизить риск, что человека не ознакомили. Это общий документооборот компании, не отдельная система службы охраны труда. Инициатор не назван.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="252" customHeight="1">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Блок 3. СЭД и информационная среда</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Расскажите, пожалуйста, как в вашей организации устроена работа с СЭД, которую вы используете для документов по охране труда.
+Уточнения: Какую систему вы используете? Когда и в связи с чем она появилась? Для каких задач первоначально внедрялась?</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Одной системы для охраны труда нет. Звучат: КЭДО для утверждения документов, приказов и ознакомления; отдельные системы на разных предприятиях; всё ещё внедряемый SAP; контур, который в расшифровке звучит как «ЭРА»; местами 1С; TESSA для согласования ЛНА и организационно-распорядительных документов; учёт проверок и происшествий по регионам, который, по их оценке, отлажен. Название «система 12» и аббревиатура «КС» в записи не раскрыты. Когда именно появилась каждая система, не сказано. КЭДО используется не только для охраны труда: через него же отпуска, командировки и заявки.</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Своя автоматизированная система управления охраной труда и промышленной безопасностью, полностью собственная разработка. На рынке смотрели 1С по охране труда и других поставщиков и нужный набор не получили. Система частично интегрирована с корпоративной 1С и с общим документооборотом компании: что-то забирает и что-то отдаёт, не всё. Основной учёт охраны труда на их платформе. Часть операций вынесена в мобильное приложение. Первоначально система собирала журналы, предписания, инструктажи, наряды-допуски и производственный контроль, а не только подпись.</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Отдельная СЭД охраны труда не названа. Есть единый личный кабинет, фраза о платформе почти не разобрана. Есть свой удостоверяющий центр. Классический документооборот — договоры и доверенности. Кадровые документы подписываются по регламенту с коротким сроком на согласие и с санкцией, если человек не успел; срок в одном месте звучит как «полгода», контекст неясен, цифру как факт не фиксирую. Много самописных функциональных систем, они плохо стыкуются. Медосмотры вынесены отдельно и пока ручные. По подрядчикам есть медицинская система, куда стекаются результаты допусков, без подписей, и пропуск на месторождение: карта, доступ есть или нет. Эту пропускную систему разрабатывали не сами. Полный текст — в файле Word этой компании.</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Название СЭД не прозвучало. Есть личный кабинет с электронной подписью для отпусков, командировок и других кадровых документов. Обучение с 2023 года ведёт провайдер. Свой контур для них важнее внешней площадки: даже подписание на соседней внутренней платформе упирается в открытую и закрытую части ключа, фраза здесь обрывочная. Когда появился кабинет, не сказано. Госключ для этих документов не используется.</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Имени СЭД охраны труда нет. Есть система видеоинструктажа: вводный туда заносят и печатают. С 2025 года есть мобильное приложение и смартфоны, которые выдают на смену, не в личное пользование. Вход — учётная запись и пароль, для наряда-допуска носитель и пропуск информационная безопасность отклонила. Телефон пишет лог у себя и отдаёт его, когда появляется связь. Кадрового ЭДО нет. Старая система названа неразборчиво.</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Для приказов и ознакомления используют КЭДО. Руководитель утверждает документ, дальше его отправляют на ознакомление. Своя это разработка или купленная, в записи не сказано. Когда система появилась и для каких задач её брали сначала, не сказано. Стационарные компьютеры, по одной реплике, не выдают, подпись идёт через корпоративный контур.</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Имя системы не названо. Есть корпоративный ЭДО, положение о нём и сервер, где всё хранится. Отдельное хранилище не заводили. Когда система появилась и для каких задач её покупали, она не знает: «честно не знаю», знает только, что сервер есть. Сейчас через неё знакомят с локальными актами и начинают инструктажи.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="182" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Блок 3. СЭД и информационная среда</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Расскажите, пожалуйста, как в вашей организации устроена работа с СЭД, которую вы используете для документов по охране труда.
+Уточнения: Как принималось решение о выборе системы? Что было наиболее важным при выборе? Учитывались ли при выборе или внедрении системы особенности документов по охране труда? Какие именно?</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Итогового выбора системы под охрану труда ещё нет: в этом году рассчитывают открыть проект и сначала описать процессы верхнего уровня. Важное, что они сами называют: не вложить деньги и потом получить требование выгружать документы в госключ; ничего не хранить на внешних ресурсах; простой интерфейс, мало кнопок и полей. Особенности охраны труда в выборе звучат как мобильный персонал, карьер без связи, наряд, спецодежда, стажировка и наставник, а не как формальный чек-лист при закупке.</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Покупные системы не закрыли пакет, который они хотели завести в компанию, поэтому написали свою. Важными были прозрачность по всей массе работников, скорость, контроль сроков и возможность работать не только с компьютера. Особенности охраны труда закладывали сразу: инструктажи, наряд-допуск, предписания, производственный контроль, пожарный инструктаж, роли выдающего и допускающего. Отдельного протокола тендера он не пересказывал.</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Историю выбора СЭД под документы охраны труда не рассказали. По кадровому и договорному контуру важно другое: квалифицированная подпись, флешка-токен, свой удостоверяющий центр, а не госключ. Госключ он оценивает как «нам точно не надо». Особенности охраны труда на выбор системы не повлияли, потому что самого выбора под эти документы в записи нет: мешает периметр и то, что рабочие не у компьютера.</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Как выбирали систему, не рассказано. Наиболее важное, что он повторяет уже по итогам: не привязывать работодателя к одному ресурсу и не заставлять компанию, у которой система есть, жить в чужой. Особенности документов охраны труда при выборе в записи не фигурируют. Для наряда-допуска они сами делят процесс на наряд и допуск, это уже настройка, а не история закупки.</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Закупку отдельной СЭД под охрану труда не описывали. Выбор, который реально проговаривался, — с информационной безопасностью: для наряда оставили ввод пароля, без физической карты и без пропуска, хотя пароль можно передать. Корпоративный смартфон вместо личного — из-за данных и потому, что объект критический. Особенности охраны труда учтены так: подпись на месте, а не в кабинете, и работа без постоянного интернета. Когда появилась платформа, не сказано.</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="196" customHeight="1">
+      <c r="A7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Блок 3. СЭД и информационная среда</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Расскажите, пожалуйста, как в вашей организации устроена работа с СЭД, которую вы используете для документов по охране труда.
+Уточнения: Все документы по охране труда проходят через эту систему или для отдельных документов используются другие информационные системы? Какие?</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Не все. Ознакомление и часть приказов идут через КЭДО. Согласование ЛНА — через TESSA, и там, по их словам, нет электронной подписи. На предприятиях остаются свои системы, SAP и 1С. Учёт происшествий и проверок — отдельный. Обучение и спецоценка со внутренним контуром связаны частично: «привязали КС, сейчас привязываем», что такое КС, не расшифровано. Между юридическими лицами договоры ходят через Астрал или Контур.Диадок; для документов охраны труда этот канал не описан.</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>По охране труда основной оборот он относит к своей системе, но не весь и не без бумаги. Рядом корпоративный документооборот и 1С, интеграция неполная. Инструктажи по охране труда и целевой инструктаж на работы повышенной опасности дублируются живой подписью. Протокол проверки знаний ещё дублируется, дубль собираются отменить. Спецоценка пока с живой подписью, результаты им подгружает внешняя организация. Журнал трёхступенчатого контроля и регистрация нарядов-допусков живут в системе без отдельной подписи.</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Нет. Сведения о новых позициях и результатах спецоценки уходят в кадровые системы, сами документы охраны труда компания в одной СЭД не проводит. Медосмотры — отдельное направление, вручную, «большая боль», со охраной труда по процессам не сшиты. Функциональные системы самописные, «скрепка», ничего лишнего в них сделать нельзя. Пропуск и медицинские данные подрядчиков — ещё один контур, без подписей.</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Нет. Кадры — в личном кабинете. Обучение — у провайдера. Спецоценка — отдельный тяжёлый процесс подписи комиссии. Наряд-допуск только переносят в электронный вид в этом году, и уже делят на два процесса. Инструктажи в корпоративную систему он не ставит. Другие имена систем не названы.</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Нет одной системы. Видеоинструктаж, приложение нарядов, бумажные журналы и сканы спецоценки живут рядом. Кадровый ЭДО документы охраны труда не покрывает. Интеграции «системы объезда» не достроены, фраза об этом обрывочная. Другие имена он не называет.</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Не все. Через КЭДО идут утверждение приказов и ознакомление с локальными актами. Личные карточки туда ещё не доведены. Инструктажи в КЭДО подписывают не всегда: «не успевают». Целевой инструктаж в разговоре отделяют от первичного и повторного. Спецоценка в эту же систему целиком не встаёт: опции приложить файл подписи эксперта к карте нет. Другие имена систем, кроме неясного блока 1С, не названы.</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Не все. Локальные акты идут через этот ЭДО. Инструктажи переводятся частично: для сторонних вводный только лично, не через ЭДО; своим работникам периодические, повторные и вводные уже ставят в систему, но вводный день в день система настраивает плохо. Целевой инструктаж редкий. Спецоценка и обучение электронно до конца не выстроены, она сама говорит, что текущая схема нарушает закон об электронной подписи. Других систем она не называет.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="238" customHeight="1">
+      <c r="A8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Блок 3. СЭД и информационная среда</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Расскажите, пожалуйста, как в вашей организации устроена работа с СЭД, которую вы используете для документов по охране труда.
+Уточнения: Есть ли документы, которые вы хотели бы перевести в электронный формат, но система пока не позволяет этого сделать? Были ли документы, которые наоборот удалось перевести в ЭДО именно благодаря возможностям системы?</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Хотят, но система пока не даёт сквозной наряд: чтобы подтянулись заявка на спецодежду, срок стажировки и наставник. Сейчас это сбор в Excel, автоматизацией они это не считают. По спецоценке в их контуре нет опции приложить файл подписи эксперта к той же карте, фраза об этом обрывочная. Удалось перевести ознакомление с локальными актами в КЭДО и на части предприятий выдавать электронное задание с идентификацией по карте.</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Технически готовы подписывать целевой инструктаж на наряде-допуске через УНЭП и пока этого не делают: ждут, можно ли так вообще, и уже много вложили. Спецоценку целиком в электронный вид не перевели: живая подпись остаётся, смена поставщика затормозила договорённость, что комиссия и работники подпишут УНЭП, а исполнитель подпишет у себя и передаст результат в портал. Госключ работникам хотят, это ещё проработка. Благодаря системе ушли от бумажного журнала трёхступенчатого контроля, собирают отчёт производственного контроля на любую дату, ведут предписания с закрытием, пожарный инструктаж подписывают УНЭП, протокол проверки знаний формируется автоматически.</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Хотели бы быстрее знать вредность и не ждать результат спецоценки до 12 месяцев: смежная служба уже требует назначенное рабочее место, класс условий сидит в мотивации, из-за лага они, по его словам, не дожидаются результата и потом пересчитывают прошедший год. В системах это не лечится, интеграции нет. Хотели бы, чтобы человек на входе прикладывал карту и видел, что ему нужно сделать, не выходя во внешнее решение. Что именно удалось перевести в ЭДО благодаря системе, по охране труда не названо. В кадровом контуре задание на согласие до работника доходит.</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Вводный инструктаж и вообще инструктажи в предложенной внешней модели он не видит, как реализовать: нужно ещё согласие на электронный оборот. Наряд-допуск хотят в этом году, наряд — полностью электронное согласование; что будет с допуском, фраза обрывается. Благодаря кабинету кадровые документы уже подписываются без госключа. Обучение ушло к провайдеру. Что система технически не умеет, кроме этой развилки, не сказано.</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Хотели бы не дублировать допуск, но не вошли в эту схему: смотрели опыт, где бумагу уже не ведут, и сами туда не пошли. Вводный можно было бы не печатать, но они печатают и подписывают от руки. Система видеоинструктажа как раз позволила заносить вводный и печатать его из системы, а не вести только журнал. Кадровые документы система не возьмёт ещё несколько лет из-за смены версии. Цифровизацию как тему он в разговоре про обучение готов отложить.</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Да. Личные карточки проект ещё не закрыл. По спецоценке систему нельзя заставить приложить к карте файл подписи эксперта, опции нет, это надо настраивать. Протокол проверки знаний они не собирают как один оригинал на весь южный дивизион. Благодаря КЭДО уже идёт ознакомление с набором документов по должности, и есть кнопка вернуть документ на подписание.</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Да. Вводный инструктаж своим работникам не всегда проходит в тот же день, система не донастроена. В результат попадает тот, кто назначил инструктаж, а не руководитель, который его провёл, и сам руководитель в моменте не подписывает. Спецоценку и обучение нельзя честно считать электронными, пока внешняя организация не пришлёт документ, подписанный электронно, а не скан с живыми подписями. Благодаря системе получилось массовое ознакомление с отбором по человеку, должности и подразделению и повторные напоминания.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="210" customHeight="1">
+      <c r="A9" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Блок 3. СЭД и информационная среда</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Расскажите, пожалуйста, как в вашей организации устроена работа с СЭД, которую вы используете для документов по охране труда.
+Уточнения: Что в СЭД сегодня больше всего помогает работе с документами по ОТ, а что создаёт сложности? Можете привести конкретный пример?</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Помогает КЭДО: ежедневное напоминание о подписании, аннулирование, если срок прошёл, выгрузка документа и файлов подписей, отметки, кто подписал, уведомление на компьютер и на телефон, возможность не подписать и написать, что не устраивает. Для проверки можно отфильтровать неподписавших и новичков. Мешает TESSA: подписи нет, фильтров и кнопок так много, что работник, по их словам, потеряется. Процессы не связаны: непройденное обучение само в связанный контур не подтягивается. Название КЭДО в одном месте звучит неразборчиво, похоже на «КОТ».</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Помогает прозрачность: видно, где по более чем 35 тысячам человек просрочен любой вид инструктажа, кто выписал несоответствие и кто его закрыл, система напоминает о сроке. В мобильном приложении можно приложить фото устранения. Сложность, которую он сам называет непобеждённым барьером, — подпись. Плюс связь глушат в приграничных регионах, а часть возрастных работников остаётся на кнопочных телефонах. Правила электронного оборота пока разбросаны по разным документам, единого стандарта нет.</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Для охраны труда помощь СЭД почти не из чего складывать: электронного ознакомления нет. В кадровом контуре помогает то, что задание приходит само, срок короткий, токен спрашивается только на нужном шаге, а не висит открытым. Сложности: рабочий не онлайн, на удалённых площадках программа открывается очень медленно, даже стационарные телефоны местами убрали и оставили внутреннюю связь, системы не стыкуются, поддержка любой новой системы стоит отдельных людей. Пример — разрыв спецоценки и кадров на 12 месяцев.</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Самым сложным процессом он называет подписание комиссией результатов спецоценки: нужно пройтись по людям, уходит много времени. Остальные сложности — технические и организационные, без примера системы, которая зависает. Сопротивление людей почти сошло: сейчас, по его оценке, около одного процента. Помощь системы он иллюстрирует не охраной труда, а тем, что без электронной подписи человек не получит машину и не завершит согласия.</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Помогает фиксация на месте: инструктор не кабинетный, отметка пишется в телефон и уходит в систему, когда аппарат попадает в сеть. Это для него надёжнее журнала, который потом уничтожают по сроку. Мешает отсутствие интернета и даже электричества на объекте, один объект Кольского филиала без нормальной связи, сменный телефон и пароль, который можно сказать другому, и то, что кадрового ЭДО не будет, пока группа меняет платформу. Юридически «можно и так, и по-другому» не даёт опереться на систему и выкинуть бумагу.</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>Помогает цепочка КЭДО: после подписи руководителя документ уходит на ознакомление, неподписанное можно вернуть на подписание. Мешает объём и география. В южном дивизионе одна комиссия на 50 городов, люди не успевают подписать в КЭДО, а дату в дату им нужно. По спецоценке удалённость мешает очному ознакомлению, а система не принимает файл подписи. Пример с тысячей пунктов выдачи они приводят сами: одну инструкцию нельзя размножить в тысячу оригиналов.</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Помогает рассылка по нужной группе, круглосуточный доступ, фиксация времени подписи и напоминание, что подошёл срок повторного ознакомления. По ощущению сильно меньше ручной работы и ниже риск пропуска. Сложности в основном на старте: систему надо настроить, это занимает время. Дальше серьёзных проблем она не описывает. Работники спрашивают, куда нажать: не у всех, по её словам, хватает навыка. Фраза, висит ли система при большом объёме, противоречивая, вывода о сбоях не делаю.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="252" customHeight="1">
+      <c r="A10" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Блок 4. Общая карта документов</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Какие документы по ОТ у вас сегодня полностью существуют и обращаются в электронной форме?
+Уточнения: Почему именно эти документы?</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Полного списка нет. В электронном виде ходят ознакомление с локальными актами и утверждение приказов и документов в КЭДО. На части предприятий есть электронное задание с идентификацией по карте. Почему эти: много людей, текучка и перестановки, без системы это не проконтролировать.</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Полностью без бумаги и без живой подписи он описывает журнал трёхступенчатого контроля и регистрацию, открытие и закрытие наряда-допуска: достаточно учётной записи и роли. Предписания производственного контроля и сбор отчёта тоже идут в системе, отчёт затем отдают в Ростехнадзор электронно вместе с экспертизами. Пожарный инструктаж и ознакомление с дефектной ведомостью экспертизы промышленной безопасности подписаны УНЭП. Почему так: пожарный инструктаж, по его словам, не попадает под ограничения приказа об обучении по охране труда, а трёхступенчатый контроль и регистрацию наряда они сознательно оставили на учётной записи. Полный текст — в файле Word этой компании.</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Таких документов по охране труда он не назвал. Прямо сказано, что электронно работников с этими результатами не знакомят. В электронном виде ходят сведения для кадровой системы и данные допуска подрядчиков, это не подписанный документ охраны труда.</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Полного списка документов охраны труда, которые только электронные, нет. Обучение переводят в ЭДО с 2023 года. Кадровые документы в личном кабинете электронные, это не охрана труда. Почему начали с них, он не объясняет отдельно: кадры были готовы раньше.</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Полностью электронных документов охраны труда он не назвал. Вводный есть в системе и всё равно печатается на подпись. Наряд в приложении бумагу не заменил. Спецоценку подписывали в классическом виде и сканировали.</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Полностью электронным они описывают ознакомление с локальными актами в КЭДО, блоками по должности. Почему эти: набор повторяется, а пунктов выдачи около тысячи, делать на каждый отдельный оригинал инструкции они не могут и не считают нужным. Инструктажи, протоколы и личные карточки к полностью электронным не относят.</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Полностью электронным она описывает ознакомление с локальными актами: сообщение, вход, подпись в системе. Почему они: документы общие и цеховые, адресатов много, бумага здесь как раз лишняя. Инструктажи, спецоценка и обучение к полностью электронным не относятся, бумагу по ним дублируют.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="154" customHeight="1">
+      <c r="A11" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Блок 4. Общая карта документов</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Какие документы остаются исключительно на бумаге?
+Уточнения: Почему именно эти документы?</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Закрытого списка «только бумага» нет. Бумага остаётся там, где процесса в системе ещё нет: сквозной наряд и часть спецоценки. Отдельно — площадка без связи: перед выездом на карьер подписать негде, горный мастер не сидит в кабинете. Оригиналы по спецоценке люди по-прежнему просят. Причина в записи: нет устойчивой связи, нет готового процесса и жёсткая политика информационной безопасности.</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Живая подпись остаётся на инструктажах по охране труда, на целевом инструктаже при работах повышенной опасности и на спецоценке. Бумагу по талону на нарушение из фразы однозначно не восстановить, вывод не делаю. По вахтовому крану он говорит, что законодательство не даёт убрать требование целиком, над этим работают. Другие журналы, которые нельзя отменить по закону, он упоминает, но поимённо не перечисляет.</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>На бумаге, судя по описанному контуру, остаются медосмотры и спецоценка как документ, с которым работника не знакомят электронно. Инструктажи в электронной форме не описаны. Почему: производственный персонал не имеет постоянной почты и не сидит в сети, личный телефон запрещён, часть площадок на внутренней связи без обычного телефона. Полный перечень бумажных документов не проговаривался.</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Инструктажи остаются вне электронного оформления, бумагу в целом держат из-за нестабильной позиции инспекции. Какой именно журнал или акт «только бумага», он не перечислил.</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>На бумаге остаются подпись вводного, наряды-допуски и спецоценка. Обязательную форму наряда он выделяет только для одного вида работ, в расшифровке это звучит как правила при эксплуатации, точное имя правил не разобрать; остальные формы, по его словам, рекомендательные. Почему бумага: нет однозначного разрешения, первое лицо не взяло схему без дубля, связь на объекте не гарантирована.</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Закрытого списка нет. Инструкция по охране труда для сотрудника пункта выдачи одна на все точки, листа подписи в ней нет, листы ознакомления идут отдельно. Протокол проверки знаний физически гоняют копиями, пока не соберётся комиссия. Личные карточки в электронный оборот не доведены. Спецоценку в удалённых точках бумагой и копией карты они ещё обсуждают как действующее ограничение, а не как отменённый порядок.</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Вводный инструктаж для сторонних организаций — только лично, не через ЭДО. Плюс бумажный дубль там, где электронное ознакомление они не считают единственным способом, в том числе спецоценка и обучение. Закрытого списка «никогда не сканируем» нет. Причина — сторонний человек не в их ЭДО, а по своим документам они пока не готовы оставить только файл.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="210" customHeight="1">
+      <c r="A12" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Блок 4. Общая карта документов</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Какие документы существуют одновременно в электронной и бумажной форме?
+Уточнения: Бывает ли, что полностью оформленный электронный документ всё равно распечатывается? Зачем? Кто принимает решение?</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Одновременно в двух видах прямо как регламент не описано. КЭДО умеет выгрузить документ на бумагу, если это нужно. По спецоценке обсуждали подпись эксперта и отдельное ознакомление работника со скан-копией карты; это описано как ограничение системы, а не как принятое правило «печатаем всегда». Кто решает печать, не сказано.</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Да. Семь видов инструктажей по охране труда, в том числе вводный, первичный, повторный и внеплановый, фиксируются в системе (дата, кто провёл, кому, тема), а подпись остаётся живой. Целевой инструктаж на работы повышенной опасности ведут электронно и печатают на живую подпись, эти подписи хранят 30 дней, как требуют по наряду-допуску. Протокол проверки знаний ещё дублируют и дубль отменяют. Спецоценку подгружают в систему и параллельно не ушли от живой подписи. Кто лично решает печать, не сказано: печать привязана к требованию закона, а не к выбору работника.</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Прямо не сказано, что один и тот же готовый электронный документ ещё и печатают и кто это решает. Бумага и электронный контур существуют рядом: инспекция, по его словам, не даёт спокойно оставить только электрон, а часть процессов уже не пускает человека дальше без электронной подписи.</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Да. Вводный заносят электронно и печатают на живую подпись. Наряд смотрели в электронном виде и дублируют бумагой. Спецоценка — живые подписи и скан. Кто утверждает печать, не сказано: для вводного печать встроена в порядок, для наряда они сознательно не перешли к чужому опыту без бумаги.</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Да, для протокола. Оригинал один на южный дивизион, его копируют и пересылают по 50 городам, пока комиссия не соберёт подписи. Они прямо говорят, что так нарушают правило одного документа, и всё равно оригинал не собирают. Печать из системы как запасной путь звучит обрывочно: руководителю можно было бы сформировать запись, распечатать и подписать. Кто утверждает именно печать, не сказано.</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Да, бумагу полностью дублируют, хотя ознакомление в системе есть. По спецоценке и обучению это прямо связано с тем, что электронный файл работника не заменяет подписи комиссии и эксперта. Печатается ли уже полностью подписанный электронный документ ещё раз и кто это решает, не сказано. Дубль описан как их текущее правило на переходный период, а не как разовая печать.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="196" customHeight="1">
+      <c r="A13" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Блок 4. Общая карта документов</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Есть ли документы по охране труда, которые вы хотели бы перевести в электронную форму, но пока не смогли?
+Уточнения: Расскажите о таком документе. Что именно не позволяет перевести его в электронную форму (НПА, вид ЭП, СЭД, интеграция, организационные причины)? Что должно измениться, чтобы этот документ можно было полностью перевести в электронную форму?</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Да. Сквозной наряд со спецодеждой, стажировкой и наставником — пока Excel. Инструктажи, ознакомление в поле и обучение они относят к процессам, которые надо переводить, но не хотят завязывать на внешний контур. Мешают отсутствие понятных правил, запрет выносить документы наружу, нет связи на карьере и несвязанные системы. Чтобы сдвинуться, им нужны правила до затрат, подпись внутри своей системы «нажал и подписал» и связь либо отдельный порядок для выезда.</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Да. Подпись результатов инструктажей по охране труда: пилот не разрешили. Целевой инструктаж на наряде-допуске готов к УНЭП, но они не включают его, пока нет решения, что так можно. Спецоценка упирается в живую подпись и в смену организации, которая её проводит. Внешний проект стационарного контроля Ростехнадзора они посчитали и не пошли в него: дорого собрать единое окно, проверки не отменялись. Чтобы довести свои документы, нужно признанное правилами подписание и интеграция с тем, кто подписывает спецоценку со своей стороны.</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>В электронный вид не переведён сам документ спецоценки и ознакомление работника с ним: они передают сведения и упираются в срок, в привязку вредности к рабочему месту, а не к профессии, и в системы, которые нельзя доработать. Медосмотры тоже не в общем контуре. Что должно измениться, по его логике: вредность, известная на входе по профессии, ежедневное подтверждение личности картой внутри периметра и право не выносить процесс наружу. Это его боль, а не согласованный план перевода.</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Инструктажи, в первую очередь вводный: изменение правил их обрадовало, но реализовать у себя они не смогут, если это завязано на согласие и на один внешний ресурс. Наряд-допуск не закончен, план — этот год. Спецоценка формально идёт, но подпись комиссии слишком долгая. Чтобы сдвинуть инструктаж, нужно разрешение в логике кадрового ЭДО, без обязательной площадки. Чтобы сдвинуть спецоценку, нужен иной способ собрать подписи, чем обход каждого.</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Массовые инструктажи и наряд без бумажного дубля. Мешают неоднозначные разъяснения («можно и так, и иначе»), ответственность первого лица, отсутствие кадрового ЭДО на ближайшие годы, режим критической инфраструктуры и связь. Должно измениться правило: электронная фиксация достаточна, а не один из вариантов. Плюс устройство и канал, которые информационная безопасность пустит на объект.</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Да. Личные карточки: проект не закончен. Протокол: нельзя честно оставить один электронный документ, пока комиссия разъезжает по 50 городам и подписывает копии. Спецоценка: нет опции приложить файл подписи, а из-за удалённости с картой знакомят копией. Инструктаж на наряде-допуске они не ждут быстрым: если людям придётся ещё писать причины, в разговоре звучит, что этого скорее не сделают. Чтобы сдвинуться, нужна настройка системы под файл подписи и правило, которое не требует тысячу оригиналов и очный сбор комиссии.</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Инструктажи: система не держит день в день и не фиксирует реального руководителя. Спецоценка и обучение: нельзя перевести честно, пока нет электронно подписанного оригинала от внешней организации, скан плюс подпись работника она признаёт нарушением. Когда снимут ограничение по инструктажам, пользоваться будут, но нужен переходный период, не день в день. Чтобы закрыть спецоценку, нужно запрашивать у исполнителя архив с файлами подписи, а не бумажную карту.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="252" customHeight="1">
+      <c r="A14" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Блок 5. Глубокий разбор конкретных документов</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Давайте на примере документа разберём весь его путь от создания до хранения. Расскажите, пожалуйста, как это происходит у вас на практике.
+Уточнения: Кто инициирует документ? Где он создаётся? Кто его заполняет? Кто проверяет? Кто подписывает? Кому передаётся? Где хранится? Кто имеет доступ? Что происходит, если в документе обнаруживается ошибка? Как оформляется исправление? Что происходит с предыдущей версией?</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Один документ от создания до хранения целиком не разбирали. Частично: приказ или утверждаемый документ подписывает руководитель в КЭДО, затем помощник отправляет его на ознакомление. Если человек не подписал в срок, документ аннулируется; есть возврат на повторное подписание. Выгрузить документ и подписи можно. По спецоценке карта эксперта с файлом подписи в систему не грузится, опции нет. Кто проверяет, кто имеет доступ и что происходит со старой версией при ошибке — не сказано.</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Целиком один документ с исправлением ошибки и судьбой старой версии не разобрали. Наряд-допуск: выдающий заходит под своей учётной записью и только при нужной роли, допускающий подтверждает, производитель работ вписывает бригаду и темы инструктажа, затем лист печатают на живую подпись. УНЭП на этом шаге подготовлен и выключен. Предписание производственного контроля создаёт тот, кто выявил несоответствие, закрывает ответственный, оба под своими учётными записями, чужой логин передавать нельзя. Отчёт собирается на любую дату и уходит в Ростехнадзор с приложениями. Протокол проверки знаний формируется после практики и экзамена и рассылается на ознакомление. Полный текст — в файле Word этой компании.</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Полный путь одного документа не разобран, кусок записи про наряд пропущен расшифровкой. Спецоценка: узкое место — подписи членов комиссии, обход занимает много времени; кто создаёт карту, где она хранится и как правят ошибку, не сказано. Наряд-допуск делят на наряд и допуск, наряд будет целиком в электронном согласовании. Кадровый документ в личном кабинете работник подписывает сам, иначе не двигается связанный процесс, пример — выдача машины.</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Полной цепочки с проверкой, ошибкой и старой версией нет. Вводный: заносят в систему видеоинструктажа, печатают, подписывают от руки. Наряд: смартфон на смену, работник входит под своей учётной записью паролем, событие пишется логом в телефоне, время прикладывания или отметки хранится в аппарате и синхронизируется, когда телефон попадает в сеть станции или в город. Кто создаёт наряд и кто его проверяет, не разложено. Спецоценка подписывалась на бумаге и сканировалась. Где сервер и кто смотрит архив, не сказано.</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Один документ целиком, с ошибкой и судьбой старой версии, не разобрали. Приказ: руководитель подписывает в КЭДО, затем документ уходит на ознакомление. Если работник не подписал, есть возврат на подписание. Модель «зашёл, значит подписал» они отвергли: разрешения не нашли. Протокол: дата проверки знаний может быть раньше, чем подписи членов комиссии; обсуждали, что подписи надо собрать заранее, примерно за неделю до конца срока обучения, иначе с даты в протоколе допуск уже спорный. По спецоценке работник может подписать одну карту, а эксперт подписывал весь отчёт; они хотят архив, где к нужной карте приложен файл подписи, и говорят, что такой опции нет. Полный текст — в файле Word этой компании.</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>Локальный акт: руководитель кадров или охрана труда загружает файл, выбирает фамилии, должности или подразделение, человеку приходит сообщение, он заходит и ставит подпись. Если молчит, она пишет ему сама или через линейного руководителя; руководители тоже опаздывают. Хранится в системе, на сервере компании, отдельный архив не делали. Доступ у работника по паролю, круглосуточно, с рабочего компьютера, телефона или из дома. Инструктаж: она назначает, система запоминает назначившего, а не того, кто провёл; подпись односторонняя, руководитель в моменте не подписывает. Что делают с ошибкой и со старой версией, не сказано.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="210" customHeight="1">
+      <c r="A15" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Блок 6. Электронная подпись</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Расскажите, пожалуйста, как у вас организовано подписание документов по охране труда электронной подписью.
+Уточнения: Используется ли одинаковый подход для разных документов? Есть ли документы с особым порядком подписания?</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Одинакового порядка нет. В системе для разных процессов звучат разные типы подписей, в том числе простая. Приказ утверждается в КЭДО, ознакомление идёт отдельно, цепочкой после руководителя. Идею «зашёл в документ — значит подписал» они отвергли: разрешения на это не нашли. Особый практический узел — дата протокола проверки знаний и более поздние подписи членов комиссии: протокол одной даты, подписи другой. Как это оформляют регламентом, не договорили.</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Нет, подход разный. Большую часть внутренних записей он не считает подписью: это ознакомление и согласование под учётной записью. На прямой вопрос, не является ли это ПЭП, отвечает «нет». УНЭП используют на пожарном инструктаже (кто провёл и кто прослушал) и на ознакомлении с дефектной ведомостью экспертизы промышленной безопасности. Живая подпись остаётся на инструктажах по охране труда, целевом инструктаже и спецоценке. Протокол проверки знаний переводят на подпись со стороны компании и работника, формулировка в записи смазана.</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Для документов охраны труда единого порядка подписи нет, потому что электронного подписания этих документов не описано. В кадровом контуре порядок особый: квалифицированная подпись на флешке, пароль на вход в систему, на нужном шаге система спрашивает ключ, человек вставляет токен. Чужой токен, по его оценке, использовать не получится: надо знать систему и роль, расхождение уйдёт в безопасность. Часть кадровых форм, где бланк не закреплён законом, подписывается простой подписью; формулировка в записи смазанная. Договоры и доверенности — отдельная, более старая схема.</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Нет. Внешние управленческие и должностные документы подписывают усиленной квалифицированной подписью, её используют больше. Кадры долго жили на простой подписи, усиленная неквалифицированная — примерно последние два года, в личном кабинете, не госключом. Спецоценка — отдельный порядок из-за числа подписантов. Инструктажи электронно не подписывают.</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Одинакового порядка нет. Вводный — рукописная подпись на листе из системы. Наряд в приложении — пароль учётной записи, отдельным видом электронной подписи он это не называет. Спецоценка — живая подпись и скан. Кадровой квалифицированной подписи у них нет, контур не внедрён.</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Нет. Утверждение приказа в КЭДО и ознакомление — разные шаги, второй идёт после первого. Ознакомление они не считают автоматическим фактом входа. Протокол живёт своей датой и поздними подписями комиссии. На вопрос про одну подпись на документе по спецоценке отвечают, что так и будут делать, но как именно выровняют вид подписи, не договаривают. Целевой инструктаж подписывает охрана труда, первичный и повторный заводит руководитель.</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Нет. Ознакомление с актом — подпись работника в ЭДО. Инструктаж — односторонняя отметка, без подписи руководителя, который провёл. Спецоценка и обучение — бумажные подписи комиссии и эксперта, затем скан и электронная подпись работника. Она сама разделяет эти порядки и последний считает неправильным.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="182" customHeight="1">
+      <c r="A16" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Блок 6. Электронная подпись</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Расскажите, пожалуйста, как у вас организовано подписание документов по охране труда электронной подписью.
+Уточнения: От чего зависит вид ЭП (кто и какие виды ЭП использует)?</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Матрицы «кто каким видом подписи подписывает» компания не проговорила. Сказано, что типы подписей в системе разные и простая подпись тоже есть. Старт электронной подписи они связывают с согласием работника, в том числе при трудоустройстве; дословно согласие не зачитано. Для процессов, где факт нужно доказать, документы во внешний контур уводить не хотят.</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Вид зависит от того, считает ли компания действие подписью и что требует надзор или правило. Учётная запись — где они договорились внутри, что это фиксация роли, а не подпись. УНЭП — где надзор когда-то просил подтвердить ознакомление с экспертизой (сейчас, по его словам, уже не просит, но они оставили) и где пожарный инструктаж удалось вынести из-под ограничений обучения по охране труда. Для работников квалифицированную подпись он считает дорогой. Матрицы по должностям нет.</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>По охране труда зависимость вида подписи не задана. В кадрах вид зависит от того, зафиксирована ли бумажная форма актом: такие формы в КЭДО переводить сложно, остальное может идти простой подписью. Квалифицированный токен — у тех, кому выдали ключ и кто участвует в конкретном шаге. Рабочий персонал в эту схему не посажен.</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>От процесса. Внешнее подписание — квалифицированная подпись. Внутренние кадровые документы — подпись личного кабинета. Охрана труда на этот шаблон не посажена: комиссия спецоценки до сих пор самое долгое место, инструктажи не переведены. Кто из работников каким видом владеет, поимённо не сказано.</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>От процесса и от информационной безопасности, а не от матрицы документов. Для приложения наряда выбрали пароль, физический носитель исключили. Усиленную подпись для охраны труда он не описывает. Живая подпись остаётся там, где они не готовы отвечать за отказ от бумаги.</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Матрицы нет. Вид зависит от шага. Ознакомление в КЭДО — отдельное действие работника; простой подписью компания этот шаг не называет. Подпись руководителя на утверждении в одном месте звучит как усиленная, фраза шумная, вид подписи дословно не фиксирую. Для протокола важен не вид носителя, а то, что подписи комиссии приходят позже даты протокола. Внешних подписантов спецоценки в ту же схему они пока не посадили.</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>От документа и от того, кто вне компании. Внутреннее ознакомление закрывает подпись входа в ЭДО. Где подписантов много и они внешние, вид подписи они пока не выровняли: живая подпись остаётся у комиссии и эксперта. Матрицы по должностям нет.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="112" customHeight="1">
+      <c r="A17" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Блок 6. Электронная подпись</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Расскажите, пожалуйста, как у вас организовано подписание документов по охране труда электронной подписью.
+Уточнения: Если используется ПЭП: в какой форме используется ПЭП (код из СМС или почты, логин и пароль от корпоративной системы, логин и пароль от Госуслуг, другое)?</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Как ПЭП они учётную запись не квалифицируют и форму ПЭП не описывают. Фактически человек входит в свою учётную запись, система пускает его только при нужной роли. Код из СМС, почта и логин Госуслуг не названы.</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Словом «ПЭП» он пароль не называет. Фактически для наряда это логин и пароль корпоративного приложения на сменном смартфоне. СМС, почта и Госуслуги не используются. Пароль можно передать другому, они это понимают и всё равно остановились на пароле.</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Код из СМС, почта и логин Госуслуг не названы. По тому, как показывают ознакомление, работник в корпоративном контуре нажимает, что ознакомлен, и на этом шаге формируется отметка. Это описание процесса, а не выбранная ими формулировка «у нас ПЭП такая-то».</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>Словом «ПЭП» она подпись не называет. Практически это пароль и доступ в корпоративный ЭДО, с компьютера или с телефона, дальше подпись в системе. Код из СМС и логин Госуслуг не упоминались.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="182" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Блок 6. Электронная подпись</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Расскажите, пожалуйста, как у вас организовано подписание документов по охране труда электронной подписью.
+Уточнения: Используете ли в качестве ЭП Госключ?</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Госключ как штатный способ подписи документов по охране труда не описан. Позиция жёсткая: инструкции и документы охраны труда во внешние ресурсы не выкладывают, политика информационной безопасности это запрещает, часть сведений может быть коммерческой. Подписание в государственной системе означало бы отдать документы наружу. Продление электронной подписи через Госуслуги упоминается, это не то же самое, что подпись госключом. Фрагмент «подпись через КОТ» неразборчив.</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>В работе у работников госключа нет. Госключ хотят, и это пока проработка, не внедрение. По порталу «Работа в России» позиция компании: нельзя навязать любое готовое решение, интеграция будет трудоёмкой.</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Нет. Свой удостоверяющий центр есть, госключ он считает неподходящим: «нам точно не надо». Работник не будет подписывать документы госключом на том устройстве, которое стоит на площадке. Либо госключ, либо свой центр — развилка, которую он проговаривает, и компания остаётся при своём центре.</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Для внутренних кадровых и, судя по контексту, охрано-трудовых документов госключ не используют. Им пользуются, когда зависают Госуслуги и нужно взаимодействие с Социальным фондом и другими государственными сервисами. Он считает эту подпись тоже личной. Упрощённая процедура госключа «у ребят» упомянута неразборчиво, как устроен допуск, не восстановить.</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Нет. На вопрос про госключ на несменном личном устройстве он отвечает, что схема и так усложнённая: даже корпоративный смартфон дался тяжело, люди на смене меняются, личный телефон они не используют. Внедрения госключа нет.</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="196" customHeight="1">
+      <c r="A19" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Блок 6. Электронная подпись</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Расскажите, пожалуйста, как у вас организовано подписание документов по охране труда электронной подписью.
+Уточнения: Возникают ли сложности с подписанием электронных документов ЭП? Есть ли документы, в отношении которых сложности с электронной подписью мешают полностью перейти от бумаги к электронному документообороту? Можете привести пример?</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Да, и из-за этого бумага не уходит. Нет нормативной базы, правила приходится задавать самим. Если позже обяжут госключ, уже потраченные на свою схему деньги окажутся лишними. Отдельно: несколько усиленных подписей на одном документе и как показать их внешнему получателю; протокол одной даты и подписи комиссии другой; к карте спецоценки не приложить файл подписи; на карьере нет связи; устройство может погибнуть при аварии. Пока срок не вышел, неподписанный документ в КЭДО аннулируется — для допуска по дате это тоже риск.</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Да. Подпись он называет барьером, который пока не победили, хотя мобильное приложение уже работает. Инструктажи по охране труда из-за этого не отрываются от живой подписи. Целевой инструктаж готов к УНЭП и сознательно не включён. Людей приходится отдельно готовить: собрания, ролики, газета, видеообращения руководителей, зачем подписывать. Канал, который в расшифровке звучит как «чарлин», не восстанавливаю. Связь в приграничье рвётся, поэтому подпись с телефона не везде сработает.</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Да. Токен и компьютер не совпадают с тем, где находится рабочий: чтобы подписать, нужно прийти, открыть нужную систему и вставить флешку. Уход от стола требует блокировки, оставленный ключ — риск, хотя просто так чужой флешкой он подписать не ждёт. Для охраны труда это закрывает перевод. Госключ проблему не снимает, а выносит документ наружу, чего они не хотят. Отпуска и командировки он не комментирует, это другие коллеги.</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Да. Спецоценка упирается в то, что комиссию нужно обойти и собрать подписи, это мешает считать процесс лёгким. Подписание на другой платформе даже внутри компании сложно из-за устройства ключа. Сбои Госуслуг уводят их в госключ на государственных сервисах, не в охране труда. Из-за этого инструктажи они не обещают перевести, а бумагу держат, пока позиция инспекции нестабильна.</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Да. Пароль на общем телефоне можно передать, постоянной сети нет, поэтому подпись не онлайн, а отложенным логом, и он сам говорит, что отложенную передачу могут не принять. Пока это не признано, бумажный дубль не снимают. Отдельный пример, почему одной бумаги мало: при расследовании не нашли журнал инструктажа на рабочем месте, его уничтожили по сроку хранения. Это не сбой электронной подписи, но это причина не верить, что бумага сама по себе сохранит факт.</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Да. Люди не успевают подписать в КЭДО, а дата нужна день в день. Протокол одной даты и подписи комиссии другой ломают срок обучения. Разные виды подписи на одном документе они сами упирают в спецоценку: скан с живой подписью и электронная подпись работника вместе, по смыслу разговора, документ не собирается. Файл подписи эксперта система не принимает. Из-за этого удалённые точки остаются на копиях, а не на одном электронном оригинале.</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>Да. Люди не понимают, куда нажать, и на это уходит время. Инструктаж не подписывает тот, кто его провёл. Вводный своим нельзя стабильно провести в тот же день. Спецоценка и обучение упираются в разные виды подписи на одном документе, из-за этого бумагу не убирают. Пример она приводит сама: карта подписана от руки, её сканируют, работник подписывает электронно, так делать нельзя.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="252" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Блок 7. Электронное ознакомление</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Расскажите, как у вас организовано электронное ознакомление работников с документами по охране труда.
+Уточнения: С какими документами знакомятся электронно? Как работник получает документ? Как подтверждается ознакомление? Как фиксируются дата и время? Что происходит, если работник не ознакомился? Как организуется массовое ознакомление? Как работаете с персоналом, который не имеет постоянного доступа к компьютеру? Есть ли документы, с которыми вы не можете организовать полноценное электронное ознакомление, хотя хотели бы это сделать? Почему?</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Электронно знакомят с локальными актами. Работнику приходит задача в КЭДО, он подписывает. Не подписал — напоминание каждый день, затем аннулирование; можно вернуть на подписание и можно отказаться, написав причину. Массовая рассылка идёт после подписи руководителя. Дата и время именно ознакомления отдельной фразой не названы, фиксируется срок и факт просрочки. Для обязательной фиксации в поле устройства собираются закупать; личный телефон годится, чтобы посмотреть нормы и обучение в личном кабинете, но не как норма для обязательной подписи. Интерфейс должен быть простым. Полноценно не получается ознакомить там, где нет связи перед выездом на карьер. Полный текст — в файле Word этой компании.</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Электронно доводят протокол проверки знаний, пожарный инструктаж и ознакомление с дефектной ведомостью. По инструктажам охраны труда в системе есть факт, но не подпись работника. Сообщение приходит на компьютер или в мобильное приложение, человек подтверждает под учётной записью либо подписывает УНЭП. Дата инструктажа фиксируется; про часы и минуты подписи отдельной фразы нет. Если срок устранения или контроля прошёл, система напоминает. Массово это закрывает более 35 тысяч человек. У кого нет смартфона, есть компьютерные классы: таких остались единицы, в основном возрастные с кнопочными телефонами. Дома пользоваться можно. Полный текст — в файле Word этой компании.</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Электронного ознакомления работников с документами охраны труда нет: «электрон нет, мы не знакомы», в кадры уходят сведения. Как работник получил бы документ, как ставится время и что будет, если не ознакомился, для охраны труда не описано. Массовое ознакомление не организовано. Почты у рабочих нет, онлайн они не сидят, личные телефоны нельзя. Карта, которой человек отмечается на табло, — желаемая схема и практика, которую он видел у энергетиков и у подрядного пропуска, а не действующее ознакомление с инструкцией. Документы, которые хотели бы так знакомить, — результаты, завязанные на рабочее место и допуск, но внешнего решения им нельзя.</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Как именно работник знакомится с документом охраны труда, не рассказано: ни канал, ни фиксация времени, ни последствия, если человек не открыл документ. Рабочему персоналу устройства, по обрывочной фразе, скорее не выдают; сам он корпоративным пользуется только для теста. Есть места, где интернета нет, при этом по восьми заводам в крупных городах связь в целом есть, противопоставление в записи смазано. Сопротивление переходу с рукописной подписи было выше, сейчас около одного процента. Часть не охрано-трудовых процессов просто не пускает дальше без электронной подписи. Полноценного электронного ознакомления с инструктажами нет.</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>С вводным знакомят через видеоинструктаж, подтверждение — подпись на распечатке. На месте отметка может лечь в телефон и уйти позже, когда аппарат в зоне связи; так он описывает и удалённую точку. Дата и время пишутся в лог телефона в момент отметки, на сервер попадают не сразу. Что будет, если человек не отметился, не сказано. Массовое ознакомление не запускали: «зачем мне это вводить», пока инструктаж как электронный процесс не принят. Компьютера у работника на объекте нет, вместо него сменный смартфон. Полноценно не ознакомить электронно те инструктажи, которые они не переводят, и любой факт на Кольском объекте, пока человек не дойдёт до связи.</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Электронно знакомят с локальными актами по должности: блок уже загружен и поднимается при приёме и переводе. Человеку приходит документ в КЭДО, он отмечает ознакомление. Если не подписал, документ можно вернуть на подписание. Дата и время отдельной фразой не названы. Массово это один и тот же набор, а не тысяча разных оригиналов: инструкция для пункта выдачи одна на все точки, лист ознакомления отдельно, в инструкции нет места для подписи. Что будет, если человек так и не откроет документ, кроме возврата на подписание, не сказано. Про собственные телефоны разборчивого ответа нет. Полный текст — в файле Word этой компании.</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>Электронно знакомят с локальными актами, в том числе отдельными для складов, не со всей компанией. Человеку приходит сообщение зайти и ознакомиться, он ставит подпись. Время подписи фиксируется. Если не ознакомился, она напоминает лично или через руководителя, плюс можно настроить повтор пакета раз в три или шесть месяцев. Массово — выбором категории, должности или подразделения. Линейный персонал чаще подписывает с личного телефона. Это не обязанность: есть рабочий компьютер с паролем, можно из дома, круглосуточно, положение об ЭДО есть, запрета личного телефона нет, аналитики «кто с какого устройства» нет. Полный текст — в файле Word этой компании.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="224" customHeight="1">
+      <c r="A21" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Блок 8. Нормативное регулирование</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Были ли случаи, когда нормативное требование не позволяло организовать электронный документооборот так, как вы хотели?
+Уточнения: Были ли ситуации, когда было непонятно, допускает ли нормативное регулирование электронную форму конкретного документа? Как решали такую ситуацию?</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Да. Прямо сказано: хотим двигаться, но нормативной базы нет, правила игры определяем сами и одновременно подстраиваемся под будущие требования. Модель «открыл документ — ознакомился» отвергли, потому что не нашли, что так можно. Инструктажи и другие допускающие процедуры упираются в неопределённость, каким видом подписи и в какой системе их фиксировать. Как закрывают конкретный спорный документ, кроме отказа от сомнительной схемы, не рассказано.</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Да. Электронную подпись инструктажей по охране труда в пилоте не разрешили, поэтому факт в системе есть, а подпись бумажная. По наряду-допуску живые подписи хранят 30 дней, чтобы закрыть требование. Пожарную безопасность он вывел в электронный журнал именно потому, что ограничение обучения по охране труда на неё, по его словам, не распространяется. По вахтовому крану требование убрать нельзя, работают точечно. Где норма была неясна, они согласовывали с Ростехнадзором форму отчёта производственного контроля и вид ознакомления с экспертизой.</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Да. Бумажные формы, которые закон требует в определённом виде, в кадровый ЭДО переводятся плохо. По спецоценке закон связывает класс с рабочим местом, а бизнесу нужно понять вредность позиции раньше, чем через 12 месяцев; вакансию, по его словам, спецоценкой не закрыть. Медосмотры меняют требования и сидят отдельно. Где было неясно, они ставят «заплатки» в трудовом договоре и сами принимают решение о вредности, не дожидаясь результата. Это он сам называет разрывом и нарушением выстроенного процесса.</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Да. Бумагу оставляют, потому что позиция инспекции пока не устойчивая. На проект, который разрешал бы электронные инструктажи, они подавали комментарий: сделать так же, как по кадровому ЭДО, и не привязывать работодателя к одной системе. Иначе вводный инструктаж они не реализуют, в том числе из-за согласия на электронный оборот. Чем кончился комментарий по существу нормы, в записи не дослушано, он ищет текст своего письма.</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Да. Письмо с разъяснением, по его пересказу, звучало как «можно и так, и по-другому», поэтому на электронный допуск без бумаги они не опёрлись. В правилах по охране труда формулировка про оборот похожая, но этого им мало. Срок хранения журнала инструктажа менялся: он рассказывает про журнал 2008–2009 годов, который при десятилетнем сроке уничтожили, и при несчастном случае подтвердить инструктаж двадцатилетней давности было нечем. Требование хранить бумагу долго не помогло. Про один вид подписи на документе спецоценки он знает, свою действующую схему скана из-за этого порочной прямо не называет.</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Да. Модель «открыл документ — уже ознакомился» отвергли: запрета не нашли, но и разрешения тоже, поэтому от схемы отказались. Протокол по требованиям должен быть одним документом, с программой, датой и тем, кому проведено; копии они всё равно возят по дивизиону и говорят, что так нарушают. Риск считают низким, пока документ не запросили. Где норма была неясна, они выбирают более осторожный вариант, а не отказ от КЭДО.</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>Да. Она прямо говорит, что по спецоценке и обучению они сейчас нарушают закон об электронной подписи: один документ оказывается и с живой подписью, и с электронной. Решают пока дублем бумаги и пониманием, что нужен электронный оригинал от обучающей организации или от организации по спецоценке. По инструктажам норма не даёт им выкинуть бумагу, даже там, где система уже ведёт запись. Неясность они закрывают дублем, а не отказом от электронного контура.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="210" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Блок 8. Нормативное регулирование</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Какие требования нормативного регулирования сегодня сильнее всего ограничивают применение ЭДО документов по охране труда?
+Уточнения: Какие из них, на ваш взгляд, необходимо изменить или уточнить?</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Сильнее всего, по их словам, мешает отсутствие правил и риск, что после внедрения обяжут внешний инструмент, в первую очередь госключ и выгрузку документов наружу. Второй ограничитель — связь и мобильный персонал: страну нормальной связью они не покроют, а горный мастер не должен сидеть в кабинете. Уточнить они хотят не статью закона, а развилку: подпись внутри своей системы, без лишних действий и без раскрытия инструкций. Пока этого нет, коммерческий собственник, по их оценке, скорее наймёт людей, чем заплатит за то, чего закон прямо не требует.</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Сильнее всего держат запрет и неясность электронной подписи инструктажей и то, что без обязательного требования они не идут в дорогой внешний контур. Отдельно мешает отсутствие единого описания: электронный наряд, журнал регистрации, пожарные инструктажи и обычные инструктажи описаны кусками в разных документах, общий стандарт только собираются сделать. Что изменить: чтобы электронную фиксацию инструктажа можно было не дублировать бумагой и чтобы это не было приклеено к одному порталу, в котором не хватает функций. Конкретных пунктов актов он не перечислял.</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Сильнее всего ограничивают не одна цитата из приказа, а связка: человек не в сети, личные устройства нельзя, бумажная форма части документов, спецоценка только через рабочее место и долгий лаг. Менять, по его позиции, нужно не в сторону единого портала. Если государству нужен факт, компания готова отдавать сведения из своей системы, как уже отдаёт кадровую отчётность. Навязанный канал и госключ он просит не вводить: виды подписей и так заданы законом об электронной подписи. Конкретные пункты для правки не продиктованы.</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Сильнее всего ограничивает идея одного обязательного ресурса и цена интеграции для компании, где система уже есть, плюс неясность, примет ли инспекция электронный документ. Изменить он предлагает сам принцип: разрешить, как в кадровом ЭДО, а не назначить площадку. Для малого бизнеса государственный ресурс без своей платформы он считает нормальным. Что расписать в норме по шагам, не говорит: сотрудники привыкли к одной экосистеме, второй контур будет лишним.</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Ограничивает неясность: электронный оборот в правилах вроде допускается и одновременно официально можно оставить любой вариант. Второй ограничитель — бумажный журнал как единственное доказательство, которое ещё и уничтожается по сроку. Уточнить нужно, что электронной фиксации достаточно. Текст правки он не предлагает. По инструктажам компания приводит пример вводного, который всё равно печатают.</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Сильнее всего мешают правило одного документа и одной вида подписи там, где люди и комиссия разъеханы: 50 городов южного дивизиона и около тысячи пунктов выдачи. Второе — система не умеет приложить файл подписи к карте спецоценки. Что изменить, они списком не говорят. По смыслу реплик им нужно ознакомление без тысячи оригиналов и протокол, который не надо физически собирать. Пункты актов не назывались.</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>Ограничивают правило одной вида подписи на документ и невозможность оставить инструктаж только в электронном виде. Изменить ей нужно первое, чтобы дубль бумаги по инструктажу после переходного периода можно было снять, и практику, при которой внешняя организация отдаёт файл с подписью, а не скан. Пункты актов она не называет. Что не стоит регулировать слишком подробно, не обсуждала.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="168" customHeight="1">
+      <c r="A23" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Блок 9. Эффект от ЭДО</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Что на практике изменилось после перевода документов по охране труда в электронную форму?
+Уточнения: Трудозатраты, скорость, контроль, доступ, поиск, ошибки, хранение, взаимодействие подразделений, взаимодействие с работниками.</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Своего расчёта эффекта компания в записи не привела. Со стороны компании: в отделе охраны труда шум из-за объёма бумаги, на ознакомление уходит 21–45 документов, даже если человек смотрит текст по диагонали. В системе проще отобрать неподписавших и готовиться к проверке. Как изменились ошибки, хранение и скорость, цифрами не сказано.</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Считают эффект, чтобы обосновать систему: прозрачность, скорость, отказ от журналов, которые заказывали сотнями в типографии, и сокращение времени на оформление наряда-допуска, служебных писем и закрытие поручений. Цифр в записи нет, он обещал собрать их и отправить почтой. Качественно: линейные руководители, которые сначала сопротивлялись, теперь благодарят, что бумаги нет. Ошибки и поиск отдельными показателями не названы.</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>По документам охраны труда эффекта нет: перевода не было. Время на «дойти и подписать» они прикидывали, но он сразу упирает в стоимость поддержки и людей, которые будут вести систему: скрытая экономия не бесплатная. Эффект кадровых отпусков и командировок считать не стал, это не его функция. Коллеги, по его пересказу, экономили бумагу и ходьбу через завод, до получаса. К охране труда эти цифры не привязаны.</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Цифр эффекта по охране труда нет. Качественно: лишнюю бумагу по согласиям стараются не копить, отдельный ресурс на хранение бумажных согласий он считает избыточным, число людей в этой фразе неразборчиво и в ответ не берётся. Без электронной подписи не выдают машину. Объём приёма назван колоссальным, сравнение с другими компаниями он готов уточнить у коллег, в записи цифры нет. Скорость, ошибки и поиск по документам охраны труда не оценены.</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Эффект от перевода документов охраны труда не считали: перевода нет. Единственный практический урок про документы — бумажный журнал не спас при расследовании, потому что был уничтожен. Экономию времени на подписи он не называл.</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Расчёта эффекта нет. Качественно они описывают не «стало быстрее на столько-то», а почему бумага не масштабируется: одну инструкцию нельзя выпустить тысячей оригиналов, комиссию по 50 городам не собрать на один лист, ознакомление по должности уже уходит в КЭДО при приёме и переводе. Ошибки, поиск и хранение цифрами не оценены. Доля электронного подписания, по их словам, только начинается, цель — 100%.</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>Своего расчёта в рублях нет. По ощущениям процесс стал заметно проще, напоминания снимают риск пропустить ознакомление, ходить за подписями больше не нужно. Ошибки, архив и скорость поиска цифрами не оценены. Про сервер на десять и двадцать лет она говорит как про будущую потребность в месте, не как про уже случившуюся проблему.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="56" customHeight="1">
+      <c r="A24" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Блок 9. Эффект от ЭДО</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>А есть ли документы, при переводе которых в электронную форму практически ничего не изменилось?
+Уточнения: Почему?</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="126" customHeight="1">
+      <c r="A25" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Блок 9. Эффект от ЭДО</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Перевод какого документа в электронный формат вы считаете наиболее успешным с точки зрения полученных эффектов?
+Уточнения: Почему?</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Один документ лучшим он не назвал. Самым большим эффектом назвал сокращение времени на наряд-допуск и на служебные письма и поручения, отдельно — отказ от закупки бумажных журналов. Прозрачность инструктажей по десяткам тысяч человек для него тоже главный практический результат, хотя подпись там ещё бумажная.</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>Один документ она не выбрала. Рабочий эффект описывает на ознакомлении с локальными актами: массовая адресация, фиксация времени и повтор по сроку. Инструктажи таким успехом не называет, там как раз дыры.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="210" customHeight="1">
+      <c r="A26" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Блок 10. Проблемы и барьеры</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Если посмотреть на ЭДО документов по охране труда в целом, что сегодня является самым сложным?
+Уточнения: Какая проблема сегодня сильнее всего ограничивает дальнейший переход к электронному документообороту?</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Самое сложное для них — двигаться без правил и не потратить бюджет на схему, которую потом заменят госключом или внешним порталом. Рядом: информационная безопасность не пускает документы наружу, на карьере нет связи, системы охраны труда не связаны между собой, а в TESSA работник теряется. Дальнейший переход сильнее всего держит связка «нет нормы + нельзя вынести документ наружу + человек не у компьютера».</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Сложнее всего подпись и принятие её людьми: без большой разъяснительной кампании работники расходятся в понимании, зачем это. Дальше переход ограничивают неясность по инструктажам и нарядам-допускам, обрывы связи и то, что дорогое внешнее окно без отмены параллельных обязанностей они включать не будут. Хранение многолетних бумажных журналов как раз было причиной уйти в цифру, а не текущей проблемой системы.</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Самое сложное — производственный персонал, который не находится в сети, при закрытом периметре: личные телефоны нельзя, где-то нет даже обычной телефонной связи, только внутренняя, на удалённой площадке программа еле открывается. Второй слой — спецоценка и кадры не стыкуются, системы самописные и почти не дорабатываются, а новое внедрение сейчас упирается в деньги и людей: раньше на развитие было легче. Дальнейший ЭДО охраны труда сильнее всего держит именно отсутствие постоянного цифрового доступа у рабочих плюс запрет выйти во внешний сервис.</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Самое тяжёлое в охране труда на сегодня — собрать подписи комиссии по спецоценке. Дальше переход ограничивают один внешний ресурс и дорогая интеграция, устройства не у всех рабочих и остаточное нежелание переходить на электронную подпись, около одного процента. Инструктажи он прямо называет тем, что они не реализуют.</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Самое сложное — решиться убрать бумагу без однозначной нормы и без решения первого лица. Дальше мешают объект критической инфраструктуры, дыры связи, сменный телефон и то, что кадровый ЭДО появится нескоро из-за смены платформы. Сильнее всего дальнейший переход держит связка «норму можно прочитать трояко» и «связи на объекте нет».</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Самое тяжёлое — собрать подпись там, где людей много и они не в одном городе: пункты выдачи, южный дивизион, комиссия, которая не успевает подписать протокол в КЭДО к нужной дате. Рядом система, в которой нет опции для файла подписи по спецоценке, и личные карточки, которые проект ещё не довёл. Дальше переход держит именно это, а не отсутствие самого КЭДО: ознакомление с актами уже электронное.</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>Сложно на старте настроить систему и научить людей, куда нажимать. Дальше переход держат инструктажи — не фиксируется реальный руководитель и не всегда выходит день в день — и связка подписей по спецоценке и обучению. Пока это не закрыто, они дублируют бумагу и не считают переход законченным.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="196" customHeight="1">
+      <c r="A27" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Блок 10. Проблемы и барьеры</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Какие изменения нормативного регулирования были бы наиболее полезны для развития ЭДО в охране труда?
+Уточнения: Что, наоборот, не стоит регулировать слишком подробно и лучше оставить на усмотрение организации?</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Полезным они считают ясные правила до того, как компания потратит деньги, и возможность подписывать внутри своей системы, без выгрузки во внешний контур. Подробно загонять всех в один портал и в госключ они не хотят: инструкции наружу не отдают, а лишние действия («выгрузил, авторизовался, подписал») сводят экономию к нулю. Готового перечня «вот эти нормы изменить» нет, это собрано из разных реплик, а не ответ списком.</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Полезно разрешить электронную фиксацию инструктажей без обязательной привязки к одному внешнему ресурсу: порталу, по его оценке, не хватает функций, а интеграция любого навязанного окна дорогая. Пример, которым он это показывает, — отказ от проекта стационарного контроля Ростехнадзора: дорого, сложно, проверки не отменили, обещанных преференций не было. Что оставить на усмотрение компании, дословно не сформулировал. По смыслу — выбор своей системы и учётной записи там, где закон не требует именно подпись.</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Полезно не заставлять вести процесс на государственном ресурсе и не подменять их удостоверяющий центр госключом. Сведения, если они нужны, компания умеет отправлять из своей системы. Слишком подробно не стоит предписывать канал и носитель подписи: у них уже токен, пароль и свой центр. Привязку вредности только к рабочему месту и только по итогу длинной процедуры он тоже считает тем, что мешает жить процессам допуска. Это позиция из разговора, не текст поправок.</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Наиболее полезно разрешить электронный оборот так же, как кадровый, без привязки к одному ресурсу. Это же поддерживали, по его словам, экспертный совет РСПП и Союз напитков. Малому бизнесу можно оставить государственный вариант, чтобы не поднимать свою платформу. Подробно регулировать выбор системы и интеграцию с уже работающим контуром не стоит: у них объём большой, люди работают в одной экосистеме, чужая площадка обойдётся дорого.</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Полезно прямое правило, что результат инструктажа, зафиксированный электронно, достаточен, без формулы «можно и так, и иначе». Слишком подробно задавать носитель не стоит: у них уже работает локальный лог и поздняя синхронизация, и именно это проходит на объекте без интернета. Госключ и личное устройство он считает лишним усложнением. Это вывод из его рассказа, не список поправок.</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>Полезным для них было бы признать электронное ознакомление и один протокол без обязанности возить бумажный оригинал по десяткам городов и без тысяча копий инструкции. Слишком подробно задавать носитель они не просят. Это сборка из того, на что они жалуются, а не продиктованный текст поправок. Госключ и портал в их репликах как просьба не звучат.</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>Полезно ей такое разрешение по инструктажам, после которого бумажный дубль можно снять, пусть и не сразу: она говорит, что переходный период понадобится. Что оставить на усмотрение организации, не сказала.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="140" customHeight="1">
+      <c r="A28" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Блок 11. ЭДО в инструктажах</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Если говорить именно об оформлении результатов инструктажей по охране труда, насколько, на ваш взгляд, необходима возможность делать это в электронной форме?
+Уточнения: Если считает необходимым: что именно сегодня делает бумажное оформление неудобным или избыточным?</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Да, для них это нужный перевод. Инструктажи, ознакомление и обучение названы процессами, где много людей, текучка и перестановки, и без системы это не контролировать. Бумага неудобна объёмом: 21–45 документов на человека, подписи, горный мастер не должен возвращаться в кабинет, перед выездом на карьер подписать часто негде.</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Для них это уже необходимость: все основные инструктажи ведут электронно и упираются только в подпись. Бумага избыточна как второй контур: живая роспись, хранение 30 дней по целевому, контроль десятков тысяч людей и журналы, от которых они в других процедурах уже отказались.</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>Саму возможность он приветствует: изменение «очень обрадовало». Бумагу при этом неудобной по шагам он не разбирает. Сразу оговаривается, что вводный инструктаж и соседние процедуры они у себя не реализуют, если вместе с разрешением придут согласие на электронный оборот и один внешний ресурс.</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>Однозначного «необходимо» нет. Вводный они уже ведут в системе и всё равно подписывают на бумаге. Массово переводить остальные не начинают. Неудобство бумаги показано на уничтоженном журнале и на том, что инструктор должен зафиксировать факт на месте, а не в кабинете. При этом он спрашивает, зачем вводить то, что пока не даёт простой замены.</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>Для объёма, который они описывают, бумага уже не работает: тысяча пунктов выдачи и одна инструкция, 50 городов и одна комиссия. Инструктажи при этом в КЭДО закрыты не до конца, люди не успевают подписать. Бумагу неудобной они показывают на копиях протокола и на невозможности сделать тысячу оригиналов, а не на пошаговом разборе журнала.</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>Для них это уже нужная возможность: инструктажи в ЭДО внедряют и при снятии ограничения хотят пользоваться этим полностью. Бумажный дубль она не защищает, он временный. Что именно избыточно в бумажном листе, по шагам не разбирает: выигрыш описывает на ознакомлении — не ходить, не ловить подпись, видеть срок.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="140" customHeight="1">
+      <c r="A29" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Блок 11. ЭДО в инструктажах</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Если говорить именно об оформлении результатов инструктажей по охране труда, насколько, на ваш взгляд, необходима возможность делать это в электронной форме?
+Уточнения: Если не считает необходимым: почему, на ваш взгляд, электронное оформление результатов инструктажей не даст существенного эффекта?</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Электронная форма не даст эффекта, если её привяжут к ресурсу, в который компанию ещё надо интегрировать, и если для инструктажа нужно отдельное согласие. Люди привыкли к своей системе, приём и так большой, второй контур для крупной компании дороже, чем для малого бизнеса. Поэтому радость от разрешения у него не превращается в план перевести вводный инструктаж.</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Существенного эффекта он пока не ждёт. Цифровизацию в ряду других задач готов отодвинуть. Пока норму читают по-разному, кадрового ЭДО нет, а связь на объекте не гарантирована, электронная форма не отменяет бумагу и добавляет спор, примут ли отложенную отправку лога. Поэтому вводный они не оставляют только в системе.</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="196" customHeight="1">
+      <c r="A30" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Блок 11. ЭДО в инструктажах</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Представьте, что организация получила возможность полностью отказаться от бумажного оформления результатов инструктажей. Как, на ваш взгляд, должен выглядеть идеальный алгоритм — от момента проведения инструктажа до окончательного оформления его результата?
+Уточнения: Кто вносит сведения в СЭД? Где должен храниться результат? Кто должен иметь доступ?</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Цельный алгоритм они не продиктовали. Из того, как описывают желаемую работу: человек на месте нажимает понятную кнопку и подписывает в своей системе, без выгрузки в другую; для обязательной фиксации компании нужно выданное устройство, для просмотра сведений хватает личного кабинета; результат лежит у них, а не на внешнем ресурсе; неподписавших видно фильтром. Кто именно вносит результат инструктажа, где строка хранения и кто имеет доступ, по ролям не разложено. Для карьера без связи такого алгоритма у них пока нет.</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Отдельный «идеальный» сценарий он не рассказывал, он описывает уже собранный. Обычный инструктаж: в системе дата, кто провёл, кому и какая тема, не хватает только признанной подписи. Целевой: выдающий и допускающий действуют под учётной записью и ролью, производитель вносит бригаду и темы, подпись УНЭП вместо печати уже подготовлена. Результат хранится в их системе, доступ есть у охраны труда по всей компании и у роли на телефоне. Кто имеет право смотреть при проверке и как исправлять ошибку, не сказано.</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>Готового идеала нет, есть их контур. Отметка на месте, в сменном смартфоне, под паролем работника. Время пишется в телефон сразу, в систему компании попадает, когда аппарат видит сеть станции или возвращается в зону связи. Кто вносит текст инструктажа, не сказано. Хранение сначала в телефоне, потом у них. Кто смотрит запись при проверке, не названо. Бумагу этот контур пока не заменяет.</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>Цельный алгоритм не продиктовали. Из обрывков: руководитель заводит первичный и повторный инструктаж, целевой подписывает охрана труда; система должна напомнить; запись можно вернуть на подписание, если человек не подписал; для наряда-допуска есть опасение, что писать причины никто не будет. Где хранится результат и кто его смотрит, не сказано. Для дивизиона у них сейчас не этот алгоритм, а один оригинал и копии, пока комиссия не соберётся.</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>Цельного алгоритма она не предложила. По дырам текущей схемы ей нужно другое: инструктаж проводится в тот же день, в системе остаётся тот, кто реально провёл, а не только тот, кто назначил, работник подписывает результат, запись лежит в той же системе. Кто имеет доступ при проверке и кто вносит текст, если это не сам работник, не сказано. Это реконструкция из её претензий к системе, не отдельный проект.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="238" customHeight="1">
+      <c r="A31" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Блок 11. ЭДО в инструктажах</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Сейчас рассматривается подход, при котором оформление результатов инструктажей может быть организовано через портал «Работа в России» с идентификацией пользователя через ЕСИА. Хотелось бы узнать ваше мнение о такой модели. Как вы в целом относитесь к такому подходу?
+Уточнения: Что в такой модели может быть полезным? Какие проблемы такая модель может создать на практике (нет интернета, сбои портала, интеграция с внутренними системами, массовые инструктажи, территориально распределённые работники, работники без постоянного доступа к цифровым устройствам, личное устройство, исправление ошибки, хранение, предоставление сведений при проверке)?</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>К модели портала и госключа относятся настороженно. Полезно для них было бы не ведение процесса на портале, а чтобы человек подписал внутри компании. Проблемы, которые они называют сами: документы и инструкции нельзя выносить наружу; часть сведений коммерческая; на карьере и в разъездах нет устойчивой связи; устройство может быть уничтожено при аварии; каждое лишнее действие съедает эффект. Про сбои портала, исправление ошибки и показ сведений инспектору отдельно не говорили. Идентификацию через ЕСИА в этой реплике не разбирали.</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Отдельной оценки портала «Работа в России» он не дал. Близкая и уже прожитая позиция — внешнее государственное окно: собрать данные в одно место и отдавать их регулятору было дорого и сложно, параллельные проверки не исчезли, поэтому в проект Ростехнадзора они не пошли. Полезным такое окно он не называет. Проблемы, которые переносимы на портал инструктажей: стоимость интеграции, второй контур рядом со своей системой, нет связи в части регионов, не у всех есть смартфон. Сбои портала и показ сведений инспектору он на «Работу в России» не проецировал.</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Портал как место, где компания будет проводить инструктаж, ему не подходит: процессы туда не встроить, а государство не должно диктовать единственный способ. Про сам проект постановления он знает мало. Полезным считает только обмен данными: факт, что конкретный работник прошёл инструктаж, можно отдать из своей системы, как уже отдают кадровые сведения. Проблемы он называет своими ограничениями: нет постоянного доступа у рабочих, нет личных телефонов, слабая связь, нельзя выносить контур наружу, госключ не ложится на их удостоверяющий центр. Сбои портала отдельным примером не разбирал.</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>К одному ресурсу относится плохо. Полезно это может быть малому бизнесу, которому не надо поднимать свою платформу. Для них проблемы такие: интеграция станет очень дорогой, сотрудники живут в одной экосистеме, объём приёма большой, инструктаж упирается в согласие, Госуслуги и так иногда не работают. Интернет на восьми заводах в крупных городах в целом есть, отдельные точки без связи упомянуты неразборчиво. Массовые инструктажи, исправление ошибки и хранение на портале он не разбирал.</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>Отдельной оценки портала «Работа в России» нет. Близко к модели он говорит про отложенную выгрузку: факт фиксируется без интернета и уходит позже, а такой поздний обмен могут не принять. Госключ на сменном телефоне для него слишком сложен. Пользу единого портала он не назвал. Проблемы, которые у него уже есть и которые модель повторит: нет интернета, объект закрытый, устройство не личное и не постоянное, люди территориально на станциях, в том числе на Кольском филиале.</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="182" customHeight="1">
+      <c r="A32" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Блок 11. ЭДО в инструктажах</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Как вы относитесь к тому, что работнику потребуется идентифицироваться через ЕСИА для оформления результата инструктажа?
+Уточнения: Для каких категорий работников это может стать проблемой? Есть ли у вас работники, для которых такой способ идентификации будет затруднителен? Что делать, если работник не может или не хочет воспользоваться таким способом идентификации?</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Прямо про ЕСИА не говорили. Обязательную фиксацию они не переносят на личный телефон: для неё планируют закупать устройства, а личный кабинет на своём телефоне — чтобы смотреть нормы и обучение. Трудные категории в их рассказе — люди на карьере и разъездной персонал без связи, плюс работники, которым нужен интерфейс из минимума кнопок. Что делать, если человек откажется от ЕСИА, не сказано. В КЭДО отказ от подписи с комментарием уже есть, но это другая система.</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Про ЕСИА не говорили. Идентификация сейчас — своя учётная запись, на части задач телефон. Затруднительно это единицам с кнопочными телефонами, в основном возрастным, кто не хочет учиться: для них сделаны компьютерные классы, дома в приложении работать можно. Что делать при отказе именно от ЕСИА, не обсуждалось.</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Про ЕСИА прямо не говорили. Идентификация, которую они готовы обсуждать, — карта или токен внутри периметра, не личный телефон и не внешний сервис. Затруднительно это будет рабочим специальностям: почты нет, в онлайне они не сидят, личный телефон запрещён, на смену в других компаниях, по его примеру, выдают общее устройство. Что делать при отказе от ЕСИА, не сказано. Свой вариант — отметиться картой на месте и не выходить наружу.</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>Про ЕСИА не говорили. Сейчас работник вводит пароль в корпоративном приложении на телефоне, который выдан на смену. Пароль можно сообщить другому, это принятый компромисс с информационной безопасностью. Личный телефон не используют, даже корпоративный смартфон внедряли с сопротивлением. Категория, которой будет трудно, — смена на объекте без связи и без личного устройства. Замены ЕСИА он не предлагал.</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="168" customHeight="1">
+      <c r="A33" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Блок 11. ЭДО в инструктажах</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Если оформление результатов инструктажей будет происходить через портал «Работа в России», как, на ваш взгляд, это должно взаимодействовать с корпоративной СЭД организации?
+Уточнения: Должны ли сведения автоматически передаваться в корпоративную систему? Нужно ли организации хранить «копию» информации об инструктажах?</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Процесс они хотят оставлять в своей системе. Автоматическую передачу всего массива инструктажей на портал не поддерживают: «мы ничего не храним на внешних ресурсах». Копия, по смыслу их позиции, и есть запись в корпоративном контуре. Технической схемы обмена с «Работой в России» они не предлагали.</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Прямого ответа «забирать ли копию с портала» нет. Своя система уже место учёта, с 1С и корпоративным документооборотом она связана частично. Внешний шлюз, который они оценивали для Ростехнадзора, показался дорогим именно потому, что данные надо ещё раз собрать и отдать. Автоматическую передачу на портал как обязанность он не поддерживает. Хранить запись у себя им нужно: оттуда же контроль и отчёт.</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Взаимодействие он видит наоборот относительно портала как мастера процесса: сведения должны уходить из корпоративной системы, а не процесс — на портал. Кадровую отчётность они уже так отдают. Автоматически забирать инструктажи с «Работы в России» он не просит. Копию хранить у себя нужно хотя бы потому, что они сами называют себя точкой, которая передаёт данные в кадры и дальше живёт в своих системах. Готовой интеграции с порталом нет.</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>Чужую площадку они не хотят делать местом процесса. Даже между своими платформами подписание уже сложное. Сведения должны оставаться в их экосистеме, автоматический обмен с порталом как цель не звучит. Копия им нужна по сути как исходная запись у себя: именно в своей системе люди работают. Схему «портал главный, компания забирает копию» он не поддерживает.</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>Связки с порталом нет. Кадровой СЭД, с которой портал мог бы обмениваться, в ближайшие годы не будет, группа меняет версию платформы. Запись они видят у себя после синхронизации телефона. Нужна ли отдельная копия, прямо не сказано: фактически она сначала лежит в телефоне, затем в их контуре. Автоматическую передачу на «Работу в России» не обсуждали.</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="126" customHeight="1">
+      <c r="A34" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Блок 11. ЭДО в инструктажах</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Если бы вам поручили сформулировать требования к будущей системе электронного оформления результатов инструктажей, какие три требования вы бы поставили на первое место?</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Тремя пунктами не формулировали. Из разных реплик складываются такие условия: подпись внутри своей системы, без выгрузки и без госключа; минимум действий для работника, в том числе в поле; устойчивая связь либо понятный порядок для карьера и устройство, которое переживёт площадку. Это сборка, не дословный ответ на «назовите три требования».</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Тремя требованиями не назвал. По тому, что уже сделано и чего не хватает, для него критичны признанная подпись там, где система готова (УНЭП на инструктаже и наряде), работа с учётной записи и с телефона без отдельного ключа на каждого и отсутствие второго обязательного контура — бумаги или внешнего портала. Это сборка из его описания, не список, который он продиктовал.</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Тремя требованиями не назвал. По повторяющимся репликам для него важны: данные уходят из своей системы, а процесс на портал не переезжает; идентификация внутри периметра, без личного телефона; остаётся их удостоверяющий центр и токен, а не госключ. Это сборка, не продиктованный список.</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Тремя требованиями не назвал. По его комментарию к проекту на первом месте разрешение в логике кадрового ЭДО без обязательного единого ресурса, подпись в той системе, где люди уже работают, и интеграция, которая не стоит дороже самого перевода. Для малого бизнеса он готов оставить простой государственный вариант. Это сборка из комментария, не список из трёх пунктов.</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>Тремя требованиями не назвал. По собранному ими контуру на первом месте работа без постоянного интернета, идентификация, которую информационная безопасность пускает на сменное устройство, и правовое признание локального лога, чтобы бумагу можно было не дублировать. Это сборка, не его список.</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>Тремя требованиями она не назвала. По тому, что уже заставила систему делать и чего не хватает, для неё важны фиксация времени и факта подписи, в результате должен стоять реальный инструктор, а не только назначивший, и подпись с телефона или компьютера в той же системе, без отдельного хранилища. Это сборка, не её список.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="56" customHeight="1">
+      <c r="A35" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Блок 12. Завершение</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Если бы вам нужно было дать один совет организации, которая только начинает переводить документы по охране труда в электронную форму, что бы вы посоветовали?</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>без ответа</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:J35"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.2" footer="0.2"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;LОтветы компаний</oddHeader>
+    <oddFooter>&amp;RСтр. &amp;P из &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>